<commit_message>
add pcs/pitc & pcs/unit in vave
</commit_message>
<xml_diff>
--- a/app/templates/VAVE_Analysis_Import_Template.xlsx
+++ b/app/templates/VAVE_Analysis_Import_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lapto\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WebSource\PROMISE-APPS\promise-inventory\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2EDF9EE9-D545-4650-A74B-748FBA0F3F49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C998871E-B8D1-478B-9918-72F31A92B1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{62AADBC6-8410-49F7-A504-0FB573E6F6A1}"/>
   </bookViews>
@@ -177,7 +177,7 @@
     <definedName name="_FEB09">[2]VOLUME!#REF!</definedName>
     <definedName name="_FEB10">[2]VOLUME!#REF!</definedName>
     <definedName name="_FEB11">[2]VOLUME!#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$B$6:$AF$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet!$B$6:$AJ$67</definedName>
     <definedName name="_JAN08">[2]VOLUME!$C$6:$AA$6</definedName>
     <definedName name="_JAN09">[2]VOLUME!#REF!</definedName>
     <definedName name="_JAN10">[2]VOLUME!#REF!</definedName>
@@ -840,7 +840,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
   <si>
     <t>NO</t>
   </si>
@@ -987,6 +987,12 @@
   </si>
   <si>
     <t>VA/VE Material Analysis Master</t>
+  </si>
+  <si>
+    <t>Pcs/ Pitch</t>
+  </si>
+  <si>
+    <t>Pcs/ Unit</t>
   </si>
 </sst>
 </file>
@@ -1371,7 +1377,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1445,8 +1451,14 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1457,10 +1469,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="15" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1471,21 +1486,6 @@
     </xf>
     <xf numFmtId="15" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1499,6 +1499,18 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1507,9 +1519,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1578,13 +1587,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>18</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>495300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>404141</xdr:rowOff>
@@ -1602,7 +1611,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="30503813" y="20926425"/>
+          <a:off x="32504063" y="20926425"/>
           <a:ext cx="0" cy="1504279"/>
           <a:chOff x="63665100" y="150342600"/>
           <a:chExt cx="1016508" cy="908966"/>
@@ -1709,13 +1718,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>18</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>495300</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>10</xdr:row>
       <xdr:rowOff>404141</xdr:rowOff>
@@ -1733,7 +1742,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="30503813" y="11353800"/>
+          <a:off x="32504063" y="11353800"/>
           <a:ext cx="0" cy="1504279"/>
           <a:chOff x="63665100" y="150342600"/>
           <a:chExt cx="1016508" cy="908966"/>
@@ -2846,9 +2855,11 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="OD"/>
+      <sheetName val="HIS"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3040,6 +3051,7 @@
       <sheetName val="In Proses_IND"/>
       <sheetName val="In Proses_KRS"/>
       <sheetName val="Assumptions"/>
+      <sheetName val="_LOD"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -3229,6 +3241,7 @@
       <sheetData sheetId="53" refreshError="1"/>
       <sheetData sheetId="54" refreshError="1"/>
       <sheetData sheetId="55" refreshError="1"/>
+      <sheetData sheetId="56" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -8040,7 +8053,7 @@
   <sheetPr>
     <tabColor rgb="FFFF9900"/>
   </sheetPr>
-  <dimension ref="A1:AF67"/>
+  <dimension ref="A1:AJ67"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.33203125" style="1" customWidth="1"/>
@@ -8054,260 +8067,288 @@
     <col min="10" max="10" width="16.5546875" style="1" customWidth="1"/>
     <col min="11" max="12" width="20.6640625" style="1" customWidth="1"/>
     <col min="13" max="13" width="21.5546875" style="1" customWidth="1"/>
-    <col min="14" max="16" width="14.5546875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="17.88671875" style="1" customWidth="1"/>
-    <col min="18" max="18" width="27.88671875" style="1" customWidth="1"/>
-    <col min="19" max="20" width="34.6640625" style="2" customWidth="1"/>
-    <col min="21" max="21" width="43.44140625" style="1" customWidth="1"/>
-    <col min="22" max="22" width="20.44140625" style="1" customWidth="1"/>
-    <col min="23" max="23" width="16.21875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="16.5546875" style="1" customWidth="1"/>
-    <col min="25" max="26" width="20.6640625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="21.5546875" style="1" customWidth="1"/>
-    <col min="28" max="30" width="14.5546875" style="1" customWidth="1"/>
-    <col min="31" max="31" width="17.88671875" style="1" customWidth="1"/>
-    <col min="32" max="32" width="27.88671875" style="1" customWidth="1"/>
-    <col min="33" max="16384" width="9.109375" style="1"/>
+    <col min="14" max="18" width="14.5546875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="17.88671875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="27.88671875" style="1" customWidth="1"/>
+    <col min="21" max="22" width="34.6640625" style="2" customWidth="1"/>
+    <col min="23" max="23" width="43.44140625" style="1" customWidth="1"/>
+    <col min="24" max="24" width="20.44140625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="16.21875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="16.5546875" style="1" customWidth="1"/>
+    <col min="27" max="28" width="20.6640625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="21.5546875" style="1" customWidth="1"/>
+    <col min="30" max="34" width="14.5546875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="17.88671875" style="1" customWidth="1"/>
+    <col min="36" max="36" width="27.88671875" style="1" customWidth="1"/>
+    <col min="37" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="180" customHeight="1" x14ac:dyDescent="0.65">
+    <row r="1" spans="1:36" ht="180" customHeight="1" x14ac:dyDescent="0.65">
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="30" t="s">
+      <c r="E1" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="30"/>
-      <c r="U1" s="30"/>
-      <c r="V1" s="30"/>
-      <c r="W1" s="30"/>
-      <c r="X1" s="30"/>
-      <c r="Y1" s="30"/>
-      <c r="Z1" s="30"/>
-      <c r="AA1" s="30"/>
-      <c r="AB1" s="30"/>
-      <c r="AC1" s="30"/>
-      <c r="AD1" s="30"/>
-      <c r="AE1" s="30"/>
-      <c r="AF1" s="30"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
+      <c r="O1" s="31"/>
+      <c r="P1" s="31"/>
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="31"/>
+      <c r="T1" s="31"/>
+      <c r="U1" s="31"/>
+      <c r="V1" s="31"/>
+      <c r="W1" s="31"/>
+      <c r="X1" s="31"/>
+      <c r="Y1" s="31"/>
+      <c r="Z1" s="31"/>
+      <c r="AA1" s="31"/>
+      <c r="AB1" s="31"/>
+      <c r="AC1" s="31"/>
+      <c r="AD1" s="31"/>
+      <c r="AE1" s="31"/>
+      <c r="AF1" s="31"/>
+      <c r="AG1" s="31"/>
+      <c r="AH1" s="31"/>
+      <c r="AI1" s="31"/>
+      <c r="AJ1" s="31"/>
     </row>
-    <row r="2" spans="1:32" s="5" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:36" s="5" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
-      <c r="B2" s="25" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="26" t="s">
+      <c r="B2" s="41" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="37"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="38"/>
-      <c r="M2" s="38"/>
-      <c r="N2" s="38"/>
-      <c r="O2" s="38"/>
-      <c r="P2" s="38"/>
-      <c r="Q2" s="31" t="s">
+      <c r="E2" s="32"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
+      <c r="I2" s="33"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="33"/>
+      <c r="L2" s="33"/>
+      <c r="M2" s="33"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="33"/>
+      <c r="Q2" s="25"/>
+      <c r="R2" s="25"/>
+      <c r="S2" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="R2" s="39" t="s">
+      <c r="T2" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="S2" s="37"/>
-      <c r="T2" s="38"/>
-      <c r="U2" s="38"/>
-      <c r="V2" s="38"/>
-      <c r="W2" s="38"/>
-      <c r="X2" s="38"/>
-      <c r="Y2" s="38"/>
-      <c r="Z2" s="38"/>
-      <c r="AA2" s="38"/>
-      <c r="AB2" s="38"/>
-      <c r="AC2" s="38"/>
-      <c r="AD2" s="38"/>
-      <c r="AE2" s="31" t="s">
+      <c r="U2" s="32"/>
+      <c r="V2" s="33"/>
+      <c r="W2" s="33"/>
+      <c r="X2" s="33"/>
+      <c r="Y2" s="33"/>
+      <c r="Z2" s="33"/>
+      <c r="AA2" s="33"/>
+      <c r="AB2" s="33"/>
+      <c r="AC2" s="33"/>
+      <c r="AD2" s="33"/>
+      <c r="AE2" s="33"/>
+      <c r="AF2" s="33"/>
+      <c r="AG2" s="25"/>
+      <c r="AH2" s="25"/>
+      <c r="AI2" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="AF2" s="39" t="s">
+      <c r="AJ2" s="37" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:32" s="5" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:36" s="5" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
-      <c r="B3" s="25"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="42" t="s">
+      <c r="B3" s="41"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="G3" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="34" t="s">
+      <c r="H3" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="43" t="s">
+      <c r="I3" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="25" t="s">
+      <c r="J3" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
-      <c r="M3" s="25"/>
-      <c r="N3" s="29" t="s">
+      <c r="K3" s="41"/>
+      <c r="L3" s="41"/>
+      <c r="M3" s="41"/>
+      <c r="N3" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="29" t="s">
+      <c r="O3" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="P3" s="29" t="s">
+      <c r="P3" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="40"/>
-      <c r="S3" s="42" t="s">
+      <c r="Q3" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="R3" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="S3" s="35"/>
+      <c r="T3" s="38"/>
+      <c r="U3" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="T3" s="26" t="s">
+      <c r="V3" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="U3" s="25" t="s">
+      <c r="W3" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="V3" s="34" t="s">
+      <c r="X3" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="W3" s="43" t="s">
+      <c r="Y3" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="X3" s="25" t="s">
+      <c r="Z3" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="Y3" s="25"/>
-      <c r="Z3" s="25"/>
-      <c r="AA3" s="25"/>
-      <c r="AB3" s="29" t="s">
+      <c r="AA3" s="41"/>
+      <c r="AB3" s="41"/>
+      <c r="AC3" s="41"/>
+      <c r="AD3" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="AC3" s="29" t="s">
+      <c r="AE3" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="AD3" s="29" t="s">
+      <c r="AF3" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="AE3" s="32"/>
-      <c r="AF3" s="40"/>
+      <c r="AG3" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="AH3" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="AI3" s="35"/>
+      <c r="AJ3" s="38"/>
     </row>
-    <row r="4" spans="1:32" s="5" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:36" s="5" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="44"/>
-      <c r="J4" s="29" t="s">
+      <c r="B4" s="41"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="43"/>
+      <c r="I4" s="46"/>
+      <c r="J4" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="29" t="s">
+      <c r="K4" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="29" t="s">
+      <c r="L4" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="M4" s="29" t="s">
+      <c r="M4" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="N4" s="29"/>
-      <c r="O4" s="29"/>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="32"/>
-      <c r="R4" s="40"/>
-      <c r="S4" s="42"/>
-      <c r="T4" s="27"/>
-      <c r="U4" s="25"/>
-      <c r="V4" s="35"/>
-      <c r="W4" s="44"/>
-      <c r="X4" s="29" t="s">
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="27"/>
+      <c r="R4" s="27"/>
+      <c r="S4" s="35"/>
+      <c r="T4" s="38"/>
+      <c r="U4" s="40"/>
+      <c r="V4" s="29"/>
+      <c r="W4" s="41"/>
+      <c r="X4" s="43"/>
+      <c r="Y4" s="46"/>
+      <c r="Z4" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="Y4" s="29" t="s">
+      <c r="AA4" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="Z4" s="29" t="s">
+      <c r="AB4" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="AA4" s="29" t="s">
+      <c r="AC4" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="AB4" s="29"/>
-      <c r="AC4" s="29"/>
-      <c r="AD4" s="29"/>
-      <c r="AE4" s="32"/>
-      <c r="AF4" s="40"/>
+      <c r="AD4" s="27"/>
+      <c r="AE4" s="27"/>
+      <c r="AF4" s="27"/>
+      <c r="AG4" s="27"/>
+      <c r="AH4" s="27"/>
+      <c r="AI4" s="35"/>
+      <c r="AJ4" s="38"/>
     </row>
-    <row r="5" spans="1:32" s="5" customFormat="1" ht="99.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:36" s="5" customFormat="1" ht="99.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="B5" s="25"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="36"/>
-      <c r="I5" s="45"/>
-      <c r="J5" s="29"/>
-      <c r="K5" s="29"/>
-      <c r="L5" s="29"/>
-      <c r="M5" s="29"/>
-      <c r="N5" s="29"/>
-      <c r="O5" s="29"/>
-      <c r="P5" s="29"/>
-      <c r="Q5" s="33"/>
-      <c r="R5" s="41"/>
-      <c r="S5" s="42"/>
-      <c r="T5" s="28"/>
-      <c r="U5" s="25"/>
-      <c r="V5" s="36"/>
-      <c r="W5" s="45"/>
-      <c r="X5" s="29"/>
-      <c r="Y5" s="29"/>
-      <c r="Z5" s="29"/>
-      <c r="AA5" s="29"/>
-      <c r="AB5" s="29"/>
-      <c r="AC5" s="29"/>
-      <c r="AD5" s="29"/>
-      <c r="AE5" s="33"/>
-      <c r="AF5" s="41"/>
+      <c r="B5" s="41"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="47"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
+      <c r="Q5" s="27"/>
+      <c r="R5" s="27"/>
+      <c r="S5" s="36"/>
+      <c r="T5" s="39"/>
+      <c r="U5" s="40"/>
+      <c r="V5" s="30"/>
+      <c r="W5" s="41"/>
+      <c r="X5" s="44"/>
+      <c r="Y5" s="47"/>
+      <c r="Z5" s="27"/>
+      <c r="AA5" s="27"/>
+      <c r="AB5" s="27"/>
+      <c r="AC5" s="27"/>
+      <c r="AD5" s="27"/>
+      <c r="AE5" s="27"/>
+      <c r="AF5" s="27"/>
+      <c r="AG5" s="27"/>
+      <c r="AH5" s="27"/>
+      <c r="AI5" s="36"/>
+      <c r="AJ5" s="39"/>
     </row>
-    <row r="6" spans="1:32" s="5" customFormat="1" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:36" s="5" customFormat="1" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="6"/>
       <c r="C6" s="7"/>
@@ -8324,31 +8365,35 @@
       <c r="N6" s="9"/>
       <c r="O6" s="9"/>
       <c r="P6" s="9"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="23"/>
-      <c r="S6" s="21"/>
-      <c r="T6" s="8"/>
-      <c r="U6" s="8"/>
-      <c r="V6" s="10"/>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="11"/>
+      <c r="T6" s="23"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="8"/>
       <c r="W6" s="8"/>
-      <c r="X6" s="9"/>
-      <c r="Y6" s="9"/>
+      <c r="X6" s="10"/>
+      <c r="Y6" s="8"/>
       <c r="Z6" s="9"/>
       <c r="AA6" s="9"/>
       <c r="AB6" s="9"/>
       <c r="AC6" s="9"/>
       <c r="AD6" s="9"/>
-      <c r="AE6" s="11"/>
-      <c r="AF6" s="23"/>
+      <c r="AE6" s="9"/>
+      <c r="AF6" s="9"/>
+      <c r="AG6" s="9"/>
+      <c r="AH6" s="9"/>
+      <c r="AI6" s="11"/>
+      <c r="AJ6" s="23"/>
     </row>
-    <row r="7" spans="1:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="13">
         <v>1</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
       <c r="E7" s="22"/>
-      <c r="F7" s="46"/>
+      <c r="F7" s="26"/>
       <c r="G7" s="15"/>
       <c r="H7" s="17"/>
       <c r="I7" s="20">
@@ -8364,40 +8409,44 @@
         <v>0</v>
       </c>
       <c r="P7" s="16"/>
-      <c r="Q7" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R7" s="24"/>
-      <c r="S7" s="22"/>
-      <c r="T7" s="46"/>
-      <c r="U7" s="15"/>
-      <c r="V7" s="17"/>
-      <c r="W7" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X7" s="16"/>
-      <c r="Y7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T7" s="24"/>
+      <c r="U7" s="22"/>
+      <c r="V7" s="26"/>
+      <c r="W7" s="15"/>
+      <c r="X7" s="17"/>
+      <c r="Y7" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z7" s="16"/>
       <c r="AA7" s="16"/>
       <c r="AB7" s="16"/>
-      <c r="AC7" s="18">
-        <f>IF(ISNUMBER(SEARCH("coil", V7)), (X7*Y7*AB7*W7)/1000000, IF(ISNUMBER(SEARCH("trapezoid", V7)), (X7*Y7*((Z7+AA7)/2)*W7)/1000000, (X7*Y7*Z7*W7)/1000000))</f>
-        <v>0</v>
-      </c>
+      <c r="AC7" s="16"/>
       <c r="AD7" s="16"/>
-      <c r="AE7" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF7" s="24"/>
+      <c r="AE7" s="18">
+        <f>IF(ISNUMBER(SEARCH("coil", X7)), (Z7*AA7*AD7*Y7)/1000000, IF(ISNUMBER(SEARCH("trapezoid", X7)), (Z7*AA7*((AB7+AC7)/2)*Y7)/1000000, (Z7*AA7*AB7*Y7)/1000000))</f>
+        <v>0</v>
+      </c>
+      <c r="AF7" s="16"/>
+      <c r="AG7" s="16"/>
+      <c r="AH7" s="16"/>
+      <c r="AI7" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ7" s="24"/>
     </row>
-    <row r="8" spans="1:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="13">
         <v>2</v>
       </c>
       <c r="C8" s="14"/>
       <c r="D8" s="14"/>
       <c r="E8" s="22"/>
-      <c r="F8" s="46"/>
+      <c r="F8" s="26"/>
       <c r="G8" s="15"/>
       <c r="H8" s="17"/>
       <c r="I8" s="20">
@@ -8413,40 +8462,44 @@
         <v>0</v>
       </c>
       <c r="P8" s="16"/>
-      <c r="Q8" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R8" s="24"/>
-      <c r="S8" s="22"/>
-      <c r="T8" s="46"/>
-      <c r="U8" s="15"/>
-      <c r="V8" s="17"/>
-      <c r="W8" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X8" s="16"/>
-      <c r="Y8" s="16"/>
+      <c r="Q8" s="16"/>
+      <c r="R8" s="16"/>
+      <c r="S8" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T8" s="24"/>
+      <c r="U8" s="22"/>
+      <c r="V8" s="26"/>
+      <c r="W8" s="15"/>
+      <c r="X8" s="17"/>
+      <c r="Y8" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z8" s="16"/>
       <c r="AA8" s="16"/>
       <c r="AB8" s="16"/>
-      <c r="AC8" s="18">
-        <f t="shared" ref="AC8:AC67" si="1">IF(ISNUMBER(SEARCH("coil", V8)), (X8*Y8*AB8*W8)/1000000, IF(ISNUMBER(SEARCH("trapezoid", V8)), (X8*Y8*((Z8+AA8)/2)*W8)/1000000, (X8*Y8*Z8*W8)/1000000))</f>
-        <v>0</v>
-      </c>
+      <c r="AC8" s="16"/>
       <c r="AD8" s="16"/>
-      <c r="AE8" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF8" s="24"/>
+      <c r="AE8" s="18">
+        <f t="shared" ref="AE8:AE67" si="1">IF(ISNUMBER(SEARCH("coil", X8)), (Z8*AA8*AD8*Y8)/1000000, IF(ISNUMBER(SEARCH("trapezoid", X8)), (Z8*AA8*((AB8+AC8)/2)*Y8)/1000000, (Z8*AA8*AB8*Y8)/1000000))</f>
+        <v>0</v>
+      </c>
+      <c r="AF8" s="16"/>
+      <c r="AG8" s="16"/>
+      <c r="AH8" s="16"/>
+      <c r="AI8" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ8" s="24"/>
     </row>
-    <row r="9" spans="1:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="13">
         <v>3</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
       <c r="E9" s="22"/>
-      <c r="F9" s="46"/>
+      <c r="F9" s="26"/>
       <c r="G9" s="15"/>
       <c r="H9" s="17"/>
       <c r="I9" s="20">
@@ -8462,40 +8515,44 @@
         <v>0</v>
       </c>
       <c r="P9" s="16"/>
-      <c r="Q9" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R9" s="24"/>
-      <c r="S9" s="22"/>
-      <c r="T9" s="46"/>
-      <c r="U9" s="15"/>
-      <c r="V9" s="17"/>
-      <c r="W9" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X9" s="16"/>
-      <c r="Y9" s="16"/>
+      <c r="Q9" s="16"/>
+      <c r="R9" s="16"/>
+      <c r="S9" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T9" s="24"/>
+      <c r="U9" s="22"/>
+      <c r="V9" s="26"/>
+      <c r="W9" s="15"/>
+      <c r="X9" s="17"/>
+      <c r="Y9" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z9" s="16"/>
       <c r="AA9" s="16"/>
       <c r="AB9" s="16"/>
-      <c r="AC9" s="18">
+      <c r="AC9" s="16"/>
+      <c r="AD9" s="16"/>
+      <c r="AE9" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD9" s="16"/>
-      <c r="AE9" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF9" s="24"/>
+      <c r="AF9" s="16"/>
+      <c r="AG9" s="16"/>
+      <c r="AH9" s="16"/>
+      <c r="AI9" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ9" s="24"/>
     </row>
-    <row r="10" spans="1:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="13">
         <v>4</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
       <c r="E10" s="22"/>
-      <c r="F10" s="46"/>
+      <c r="F10" s="26"/>
       <c r="G10" s="15"/>
       <c r="H10" s="17"/>
       <c r="I10" s="20">
@@ -8511,40 +8568,44 @@
         <v>0</v>
       </c>
       <c r="P10" s="16"/>
-      <c r="Q10" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R10" s="24"/>
-      <c r="S10" s="22"/>
-      <c r="T10" s="46"/>
-      <c r="U10" s="15"/>
-      <c r="V10" s="17"/>
-      <c r="W10" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X10" s="16"/>
-      <c r="Y10" s="16"/>
+      <c r="Q10" s="16"/>
+      <c r="R10" s="16"/>
+      <c r="S10" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T10" s="24"/>
+      <c r="U10" s="22"/>
+      <c r="V10" s="26"/>
+      <c r="W10" s="15"/>
+      <c r="X10" s="17"/>
+      <c r="Y10" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z10" s="16"/>
       <c r="AA10" s="16"/>
       <c r="AB10" s="16"/>
-      <c r="AC10" s="18">
+      <c r="AC10" s="16"/>
+      <c r="AD10" s="16"/>
+      <c r="AE10" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD10" s="16"/>
-      <c r="AE10" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF10" s="24"/>
+      <c r="AF10" s="16"/>
+      <c r="AG10" s="16"/>
+      <c r="AH10" s="16"/>
+      <c r="AI10" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ10" s="24"/>
     </row>
-    <row r="11" spans="1:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="13">
         <v>5</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
       <c r="E11" s="22"/>
-      <c r="F11" s="46"/>
+      <c r="F11" s="26"/>
       <c r="G11" s="15"/>
       <c r="H11" s="17"/>
       <c r="I11" s="20">
@@ -8560,40 +8621,44 @@
         <v>0</v>
       </c>
       <c r="P11" s="16"/>
-      <c r="Q11" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R11" s="24"/>
-      <c r="S11" s="22"/>
-      <c r="T11" s="46"/>
-      <c r="U11" s="15"/>
-      <c r="V11" s="17"/>
-      <c r="W11" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X11" s="16"/>
-      <c r="Y11" s="16"/>
+      <c r="Q11" s="16"/>
+      <c r="R11" s="16"/>
+      <c r="S11" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T11" s="24"/>
+      <c r="U11" s="22"/>
+      <c r="V11" s="26"/>
+      <c r="W11" s="15"/>
+      <c r="X11" s="17"/>
+      <c r="Y11" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z11" s="16"/>
       <c r="AA11" s="16"/>
       <c r="AB11" s="16"/>
-      <c r="AC11" s="18">
+      <c r="AC11" s="16"/>
+      <c r="AD11" s="16"/>
+      <c r="AE11" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD11" s="16"/>
-      <c r="AE11" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF11" s="24"/>
+      <c r="AF11" s="16"/>
+      <c r="AG11" s="16"/>
+      <c r="AH11" s="16"/>
+      <c r="AI11" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ11" s="24"/>
     </row>
-    <row r="12" spans="1:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="13">
         <v>6</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
       <c r="E12" s="22"/>
-      <c r="F12" s="46"/>
+      <c r="F12" s="26"/>
       <c r="G12" s="15"/>
       <c r="H12" s="17"/>
       <c r="I12" s="20">
@@ -8609,40 +8674,44 @@
         <v>0</v>
       </c>
       <c r="P12" s="16"/>
-      <c r="Q12" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R12" s="24"/>
-      <c r="S12" s="22"/>
-      <c r="T12" s="46"/>
-      <c r="U12" s="15"/>
-      <c r="V12" s="17"/>
-      <c r="W12" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X12" s="16"/>
-      <c r="Y12" s="16"/>
+      <c r="Q12" s="16"/>
+      <c r="R12" s="16"/>
+      <c r="S12" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T12" s="24"/>
+      <c r="U12" s="22"/>
+      <c r="V12" s="26"/>
+      <c r="W12" s="15"/>
+      <c r="X12" s="17"/>
+      <c r="Y12" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z12" s="16"/>
       <c r="AA12" s="16"/>
       <c r="AB12" s="16"/>
-      <c r="AC12" s="18">
+      <c r="AC12" s="16"/>
+      <c r="AD12" s="16"/>
+      <c r="AE12" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD12" s="16"/>
-      <c r="AE12" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF12" s="24"/>
+      <c r="AF12" s="16"/>
+      <c r="AG12" s="16"/>
+      <c r="AH12" s="16"/>
+      <c r="AI12" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ12" s="24"/>
     </row>
-    <row r="13" spans="1:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="13">
         <v>7</v>
       </c>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
       <c r="E13" s="22"/>
-      <c r="F13" s="46"/>
+      <c r="F13" s="26"/>
       <c r="G13" s="15"/>
       <c r="H13" s="17"/>
       <c r="I13" s="20">
@@ -8658,40 +8727,44 @@
         <v>0</v>
       </c>
       <c r="P13" s="16"/>
-      <c r="Q13" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R13" s="24"/>
-      <c r="S13" s="22"/>
-      <c r="T13" s="46"/>
-      <c r="U13" s="15"/>
-      <c r="V13" s="17"/>
-      <c r="W13" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X13" s="16"/>
-      <c r="Y13" s="16"/>
+      <c r="Q13" s="16"/>
+      <c r="R13" s="16"/>
+      <c r="S13" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T13" s="24"/>
+      <c r="U13" s="22"/>
+      <c r="V13" s="26"/>
+      <c r="W13" s="15"/>
+      <c r="X13" s="17"/>
+      <c r="Y13" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z13" s="16"/>
       <c r="AA13" s="16"/>
       <c r="AB13" s="16"/>
-      <c r="AC13" s="18">
+      <c r="AC13" s="16"/>
+      <c r="AD13" s="16"/>
+      <c r="AE13" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD13" s="16"/>
-      <c r="AE13" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF13" s="24"/>
+      <c r="AF13" s="16"/>
+      <c r="AG13" s="16"/>
+      <c r="AH13" s="16"/>
+      <c r="AI13" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ13" s="24"/>
     </row>
-    <row r="14" spans="1:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="13">
         <v>8</v>
       </c>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
       <c r="E14" s="22"/>
-      <c r="F14" s="46"/>
+      <c r="F14" s="26"/>
       <c r="G14" s="15"/>
       <c r="H14" s="17"/>
       <c r="I14" s="20">
@@ -8707,40 +8780,44 @@
         <v>0</v>
       </c>
       <c r="P14" s="16"/>
-      <c r="Q14" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R14" s="24"/>
-      <c r="S14" s="22"/>
-      <c r="T14" s="46"/>
-      <c r="U14" s="15"/>
-      <c r="V14" s="17"/>
-      <c r="W14" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X14" s="16"/>
-      <c r="Y14" s="16"/>
+      <c r="Q14" s="16"/>
+      <c r="R14" s="16"/>
+      <c r="S14" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T14" s="24"/>
+      <c r="U14" s="22"/>
+      <c r="V14" s="26"/>
+      <c r="W14" s="15"/>
+      <c r="X14" s="17"/>
+      <c r="Y14" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z14" s="16"/>
       <c r="AA14" s="16"/>
       <c r="AB14" s="16"/>
-      <c r="AC14" s="18">
+      <c r="AC14" s="16"/>
+      <c r="AD14" s="16"/>
+      <c r="AE14" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD14" s="16"/>
-      <c r="AE14" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF14" s="24"/>
+      <c r="AF14" s="16"/>
+      <c r="AG14" s="16"/>
+      <c r="AH14" s="16"/>
+      <c r="AI14" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ14" s="24"/>
     </row>
-    <row r="15" spans="1:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="13">
         <v>9</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
       <c r="E15" s="22"/>
-      <c r="F15" s="46"/>
+      <c r="F15" s="26"/>
       <c r="G15" s="15"/>
       <c r="H15" s="17"/>
       <c r="I15" s="20">
@@ -8756,40 +8833,44 @@
         <v>0</v>
       </c>
       <c r="P15" s="16"/>
-      <c r="Q15" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R15" s="24"/>
-      <c r="S15" s="22"/>
-      <c r="T15" s="46"/>
-      <c r="U15" s="15"/>
-      <c r="V15" s="17"/>
-      <c r="W15" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X15" s="16"/>
-      <c r="Y15" s="16"/>
+      <c r="Q15" s="16"/>
+      <c r="R15" s="16"/>
+      <c r="S15" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T15" s="24"/>
+      <c r="U15" s="22"/>
+      <c r="V15" s="26"/>
+      <c r="W15" s="15"/>
+      <c r="X15" s="17"/>
+      <c r="Y15" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z15" s="16"/>
       <c r="AA15" s="16"/>
       <c r="AB15" s="16"/>
-      <c r="AC15" s="18">
+      <c r="AC15" s="16"/>
+      <c r="AD15" s="16"/>
+      <c r="AE15" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD15" s="16"/>
-      <c r="AE15" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF15" s="24"/>
+      <c r="AF15" s="16"/>
+      <c r="AG15" s="16"/>
+      <c r="AH15" s="16"/>
+      <c r="AI15" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ15" s="24"/>
     </row>
-    <row r="16" spans="1:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="13">
         <v>10</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
       <c r="E16" s="22"/>
-      <c r="F16" s="46"/>
+      <c r="F16" s="26"/>
       <c r="G16" s="15"/>
       <c r="H16" s="17"/>
       <c r="I16" s="20">
@@ -8805,40 +8886,44 @@
         <v>0</v>
       </c>
       <c r="P16" s="16"/>
-      <c r="Q16" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R16" s="24"/>
-      <c r="S16" s="22"/>
-      <c r="T16" s="46"/>
-      <c r="U16" s="15"/>
-      <c r="V16" s="17"/>
-      <c r="W16" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X16" s="16"/>
-      <c r="Y16" s="16"/>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="16"/>
+      <c r="S16" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T16" s="24"/>
+      <c r="U16" s="22"/>
+      <c r="V16" s="26"/>
+      <c r="W16" s="15"/>
+      <c r="X16" s="17"/>
+      <c r="Y16" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z16" s="16"/>
       <c r="AA16" s="16"/>
       <c r="AB16" s="16"/>
-      <c r="AC16" s="18">
+      <c r="AC16" s="16"/>
+      <c r="AD16" s="16"/>
+      <c r="AE16" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD16" s="16"/>
-      <c r="AE16" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF16" s="24"/>
+      <c r="AF16" s="16"/>
+      <c r="AG16" s="16"/>
+      <c r="AH16" s="16"/>
+      <c r="AI16" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ16" s="24"/>
     </row>
-    <row r="17" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="13">
         <v>11</v>
       </c>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
       <c r="E17" s="22"/>
-      <c r="F17" s="46"/>
+      <c r="F17" s="26"/>
       <c r="G17" s="15"/>
       <c r="H17" s="17"/>
       <c r="I17" s="20">
@@ -8854,40 +8939,44 @@
         <v>0</v>
       </c>
       <c r="P17" s="16"/>
-      <c r="Q17" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R17" s="24"/>
-      <c r="S17" s="22"/>
-      <c r="T17" s="46"/>
-      <c r="U17" s="15"/>
-      <c r="V17" s="17"/>
-      <c r="W17" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X17" s="16"/>
-      <c r="Y17" s="16"/>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="16"/>
+      <c r="S17" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T17" s="24"/>
+      <c r="U17" s="22"/>
+      <c r="V17" s="26"/>
+      <c r="W17" s="15"/>
+      <c r="X17" s="17"/>
+      <c r="Y17" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z17" s="16"/>
       <c r="AA17" s="16"/>
       <c r="AB17" s="16"/>
-      <c r="AC17" s="18">
+      <c r="AC17" s="16"/>
+      <c r="AD17" s="16"/>
+      <c r="AE17" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD17" s="16"/>
-      <c r="AE17" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF17" s="24"/>
+      <c r="AF17" s="16"/>
+      <c r="AG17" s="16"/>
+      <c r="AH17" s="16"/>
+      <c r="AI17" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ17" s="24"/>
     </row>
-    <row r="18" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="13">
         <v>12</v>
       </c>
       <c r="C18" s="14"/>
       <c r="D18" s="14"/>
       <c r="E18" s="22"/>
-      <c r="F18" s="46"/>
+      <c r="F18" s="26"/>
       <c r="G18" s="15"/>
       <c r="H18" s="17"/>
       <c r="I18" s="20">
@@ -8903,40 +8992,44 @@
         <v>0</v>
       </c>
       <c r="P18" s="16"/>
-      <c r="Q18" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R18" s="24"/>
-      <c r="S18" s="22"/>
-      <c r="T18" s="46"/>
-      <c r="U18" s="15"/>
-      <c r="V18" s="17"/>
-      <c r="W18" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X18" s="16"/>
-      <c r="Y18" s="16"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="S18" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T18" s="24"/>
+      <c r="U18" s="22"/>
+      <c r="V18" s="26"/>
+      <c r="W18" s="15"/>
+      <c r="X18" s="17"/>
+      <c r="Y18" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z18" s="16"/>
       <c r="AA18" s="16"/>
       <c r="AB18" s="16"/>
-      <c r="AC18" s="18">
+      <c r="AC18" s="16"/>
+      <c r="AD18" s="16"/>
+      <c r="AE18" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD18" s="16"/>
-      <c r="AE18" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF18" s="24"/>
+      <c r="AF18" s="16"/>
+      <c r="AG18" s="16"/>
+      <c r="AH18" s="16"/>
+      <c r="AI18" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ18" s="24"/>
     </row>
-    <row r="19" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="13">
         <v>13</v>
       </c>
       <c r="C19" s="14"/>
       <c r="D19" s="14"/>
       <c r="E19" s="22"/>
-      <c r="F19" s="46"/>
+      <c r="F19" s="26"/>
       <c r="G19" s="15"/>
       <c r="H19" s="17"/>
       <c r="I19" s="20">
@@ -8952,38 +9045,42 @@
         <v>0</v>
       </c>
       <c r="P19" s="16"/>
-      <c r="Q19" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R19" s="24"/>
-      <c r="S19" s="22"/>
-      <c r="T19" s="46"/>
-      <c r="U19" s="15"/>
-      <c r="V19" s="17"/>
-      <c r="W19" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X19" s="16"/>
-      <c r="Y19" s="16"/>
+      <c r="Q19" s="16"/>
+      <c r="R19" s="16"/>
+      <c r="S19" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T19" s="24"/>
+      <c r="U19" s="22"/>
+      <c r="V19" s="26"/>
+      <c r="W19" s="15"/>
+      <c r="X19" s="17"/>
+      <c r="Y19" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z19" s="16"/>
       <c r="AA19" s="16"/>
       <c r="AB19" s="16"/>
-      <c r="AC19" s="18">
+      <c r="AC19" s="16"/>
+      <c r="AD19" s="16"/>
+      <c r="AE19" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD19" s="16"/>
-      <c r="AE19" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF19" s="24"/>
+      <c r="AF19" s="16"/>
+      <c r="AG19" s="16"/>
+      <c r="AH19" s="16"/>
+      <c r="AI19" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ19" s="24"/>
     </row>
-    <row r="20" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="13"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
       <c r="E20" s="22"/>
-      <c r="F20" s="46"/>
+      <c r="F20" s="26"/>
       <c r="G20" s="15"/>
       <c r="H20" s="17"/>
       <c r="I20" s="20">
@@ -8999,40 +9096,44 @@
         <v>0</v>
       </c>
       <c r="P20" s="16"/>
-      <c r="Q20" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R20" s="24"/>
-      <c r="S20" s="22"/>
-      <c r="T20" s="46"/>
-      <c r="U20" s="15"/>
-      <c r="V20" s="17"/>
-      <c r="W20" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X20" s="16"/>
-      <c r="Y20" s="16"/>
+      <c r="Q20" s="16"/>
+      <c r="R20" s="16"/>
+      <c r="S20" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T20" s="24"/>
+      <c r="U20" s="22"/>
+      <c r="V20" s="26"/>
+      <c r="W20" s="15"/>
+      <c r="X20" s="17"/>
+      <c r="Y20" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z20" s="16"/>
       <c r="AA20" s="16"/>
       <c r="AB20" s="16"/>
-      <c r="AC20" s="18">
+      <c r="AC20" s="16"/>
+      <c r="AD20" s="16"/>
+      <c r="AE20" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD20" s="16"/>
-      <c r="AE20" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF20" s="24"/>
+      <c r="AF20" s="16"/>
+      <c r="AG20" s="16"/>
+      <c r="AH20" s="16"/>
+      <c r="AI20" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ20" s="24"/>
     </row>
-    <row r="21" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="13">
         <v>14</v>
       </c>
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
       <c r="E21" s="22"/>
-      <c r="F21" s="46"/>
+      <c r="F21" s="26"/>
       <c r="G21" s="15"/>
       <c r="H21" s="17"/>
       <c r="I21" s="20">
@@ -9048,40 +9149,44 @@
         <v>0</v>
       </c>
       <c r="P21" s="16"/>
-      <c r="Q21" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R21" s="24"/>
-      <c r="S21" s="22"/>
-      <c r="T21" s="46"/>
-      <c r="U21" s="15"/>
-      <c r="V21" s="17"/>
-      <c r="W21" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X21" s="16"/>
-      <c r="Y21" s="16"/>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="16"/>
+      <c r="S21" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T21" s="24"/>
+      <c r="U21" s="22"/>
+      <c r="V21" s="26"/>
+      <c r="W21" s="15"/>
+      <c r="X21" s="17"/>
+      <c r="Y21" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z21" s="16"/>
       <c r="AA21" s="16"/>
       <c r="AB21" s="16"/>
-      <c r="AC21" s="18">
+      <c r="AC21" s="16"/>
+      <c r="AD21" s="16"/>
+      <c r="AE21" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD21" s="16"/>
-      <c r="AE21" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF21" s="24"/>
+      <c r="AF21" s="16"/>
+      <c r="AG21" s="16"/>
+      <c r="AH21" s="16"/>
+      <c r="AI21" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ21" s="24"/>
     </row>
-    <row r="22" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="13">
         <v>15</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
       <c r="E22" s="22"/>
-      <c r="F22" s="46"/>
+      <c r="F22" s="26"/>
       <c r="G22" s="15"/>
       <c r="H22" s="17"/>
       <c r="I22" s="20">
@@ -9097,40 +9202,44 @@
         <v>0</v>
       </c>
       <c r="P22" s="16"/>
-      <c r="Q22" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R22" s="24"/>
-      <c r="S22" s="22"/>
-      <c r="T22" s="46"/>
-      <c r="U22" s="15"/>
-      <c r="V22" s="17"/>
-      <c r="W22" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X22" s="16"/>
-      <c r="Y22" s="16"/>
+      <c r="Q22" s="16"/>
+      <c r="R22" s="16"/>
+      <c r="S22" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T22" s="24"/>
+      <c r="U22" s="22"/>
+      <c r="V22" s="26"/>
+      <c r="W22" s="15"/>
+      <c r="X22" s="17"/>
+      <c r="Y22" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z22" s="16"/>
       <c r="AA22" s="16"/>
       <c r="AB22" s="16"/>
-      <c r="AC22" s="18">
+      <c r="AC22" s="16"/>
+      <c r="AD22" s="16"/>
+      <c r="AE22" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD22" s="16"/>
-      <c r="AE22" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF22" s="24"/>
+      <c r="AF22" s="16"/>
+      <c r="AG22" s="16"/>
+      <c r="AH22" s="16"/>
+      <c r="AI22" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ22" s="24"/>
     </row>
-    <row r="23" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="13">
         <v>16</v>
       </c>
       <c r="C23" s="14"/>
       <c r="D23" s="14"/>
       <c r="E23" s="22"/>
-      <c r="F23" s="46"/>
+      <c r="F23" s="26"/>
       <c r="G23" s="15"/>
       <c r="H23" s="17"/>
       <c r="I23" s="20">
@@ -9146,40 +9255,44 @@
         <v>0</v>
       </c>
       <c r="P23" s="16"/>
-      <c r="Q23" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R23" s="24"/>
-      <c r="S23" s="22"/>
-      <c r="T23" s="46"/>
-      <c r="U23" s="15"/>
-      <c r="V23" s="17"/>
-      <c r="W23" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X23" s="16"/>
-      <c r="Y23" s="16"/>
+      <c r="Q23" s="16"/>
+      <c r="R23" s="16"/>
+      <c r="S23" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T23" s="24"/>
+      <c r="U23" s="22"/>
+      <c r="V23" s="26"/>
+      <c r="W23" s="15"/>
+      <c r="X23" s="17"/>
+      <c r="Y23" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z23" s="16"/>
       <c r="AA23" s="16"/>
       <c r="AB23" s="16"/>
-      <c r="AC23" s="18">
+      <c r="AC23" s="16"/>
+      <c r="AD23" s="16"/>
+      <c r="AE23" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD23" s="16"/>
-      <c r="AE23" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF23" s="24"/>
+      <c r="AF23" s="16"/>
+      <c r="AG23" s="16"/>
+      <c r="AH23" s="16"/>
+      <c r="AI23" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ23" s="24"/>
     </row>
-    <row r="24" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="13">
         <v>17</v>
       </c>
       <c r="C24" s="14"/>
       <c r="D24" s="14"/>
       <c r="E24" s="22"/>
-      <c r="F24" s="46"/>
+      <c r="F24" s="26"/>
       <c r="G24" s="15"/>
       <c r="H24" s="17"/>
       <c r="I24" s="20">
@@ -9195,40 +9308,44 @@
         <v>0</v>
       </c>
       <c r="P24" s="16"/>
-      <c r="Q24" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R24" s="24"/>
-      <c r="S24" s="22"/>
-      <c r="T24" s="46"/>
-      <c r="U24" s="15"/>
-      <c r="V24" s="17"/>
-      <c r="W24" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X24" s="16"/>
-      <c r="Y24" s="16"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="16"/>
+      <c r="S24" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T24" s="24"/>
+      <c r="U24" s="22"/>
+      <c r="V24" s="26"/>
+      <c r="W24" s="15"/>
+      <c r="X24" s="17"/>
+      <c r="Y24" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z24" s="16"/>
       <c r="AA24" s="16"/>
       <c r="AB24" s="16"/>
-      <c r="AC24" s="18">
+      <c r="AC24" s="16"/>
+      <c r="AD24" s="16"/>
+      <c r="AE24" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD24" s="16"/>
-      <c r="AE24" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF24" s="24"/>
+      <c r="AF24" s="16"/>
+      <c r="AG24" s="16"/>
+      <c r="AH24" s="16"/>
+      <c r="AI24" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ24" s="24"/>
     </row>
-    <row r="25" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="13">
         <v>18</v>
       </c>
       <c r="C25" s="14"/>
       <c r="D25" s="14"/>
       <c r="E25" s="22"/>
-      <c r="F25" s="46"/>
+      <c r="F25" s="26"/>
       <c r="G25" s="15"/>
       <c r="H25" s="17"/>
       <c r="I25" s="20">
@@ -9244,40 +9361,44 @@
         <v>0</v>
       </c>
       <c r="P25" s="16"/>
-      <c r="Q25" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R25" s="24"/>
-      <c r="S25" s="22"/>
-      <c r="T25" s="46"/>
-      <c r="U25" s="15"/>
-      <c r="V25" s="17"/>
-      <c r="W25" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X25" s="16"/>
-      <c r="Y25" s="16"/>
+      <c r="Q25" s="16"/>
+      <c r="R25" s="16"/>
+      <c r="S25" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T25" s="24"/>
+      <c r="U25" s="22"/>
+      <c r="V25" s="26"/>
+      <c r="W25" s="15"/>
+      <c r="X25" s="17"/>
+      <c r="Y25" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z25" s="16"/>
       <c r="AA25" s="16"/>
       <c r="AB25" s="16"/>
-      <c r="AC25" s="18">
+      <c r="AC25" s="16"/>
+      <c r="AD25" s="16"/>
+      <c r="AE25" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD25" s="16"/>
-      <c r="AE25" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF25" s="24"/>
+      <c r="AF25" s="16"/>
+      <c r="AG25" s="16"/>
+      <c r="AH25" s="16"/>
+      <c r="AI25" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ25" s="24"/>
     </row>
-    <row r="26" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="13">
         <v>19</v>
       </c>
       <c r="C26" s="14"/>
       <c r="D26" s="14"/>
       <c r="E26" s="22"/>
-      <c r="F26" s="46"/>
+      <c r="F26" s="26"/>
       <c r="G26" s="15"/>
       <c r="H26" s="17"/>
       <c r="I26" s="20">
@@ -9293,40 +9414,44 @@
         <v>0</v>
       </c>
       <c r="P26" s="16"/>
-      <c r="Q26" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R26" s="24"/>
-      <c r="S26" s="22"/>
-      <c r="T26" s="46"/>
-      <c r="U26" s="15"/>
-      <c r="V26" s="17"/>
-      <c r="W26" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X26" s="16"/>
-      <c r="Y26" s="16"/>
+      <c r="Q26" s="16"/>
+      <c r="R26" s="16"/>
+      <c r="S26" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T26" s="24"/>
+      <c r="U26" s="22"/>
+      <c r="V26" s="26"/>
+      <c r="W26" s="15"/>
+      <c r="X26" s="17"/>
+      <c r="Y26" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z26" s="16"/>
       <c r="AA26" s="16"/>
       <c r="AB26" s="16"/>
-      <c r="AC26" s="18">
+      <c r="AC26" s="16"/>
+      <c r="AD26" s="16"/>
+      <c r="AE26" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD26" s="16"/>
-      <c r="AE26" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF26" s="24"/>
+      <c r="AF26" s="16"/>
+      <c r="AG26" s="16"/>
+      <c r="AH26" s="16"/>
+      <c r="AI26" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ26" s="24"/>
     </row>
-    <row r="27" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="13">
         <v>20</v>
       </c>
       <c r="C27" s="14"/>
       <c r="D27" s="14"/>
       <c r="E27" s="22"/>
-      <c r="F27" s="46"/>
+      <c r="F27" s="26"/>
       <c r="G27" s="15"/>
       <c r="H27" s="17"/>
       <c r="I27" s="20">
@@ -9342,40 +9467,44 @@
         <v>0</v>
       </c>
       <c r="P27" s="16"/>
-      <c r="Q27" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R27" s="24"/>
-      <c r="S27" s="22"/>
-      <c r="T27" s="46"/>
-      <c r="U27" s="15"/>
-      <c r="V27" s="17"/>
-      <c r="W27" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X27" s="16"/>
-      <c r="Y27" s="16"/>
+      <c r="Q27" s="16"/>
+      <c r="R27" s="16"/>
+      <c r="S27" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T27" s="24"/>
+      <c r="U27" s="22"/>
+      <c r="V27" s="26"/>
+      <c r="W27" s="15"/>
+      <c r="X27" s="17"/>
+      <c r="Y27" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z27" s="16"/>
       <c r="AA27" s="16"/>
       <c r="AB27" s="16"/>
-      <c r="AC27" s="18">
+      <c r="AC27" s="16"/>
+      <c r="AD27" s="16"/>
+      <c r="AE27" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD27" s="16"/>
-      <c r="AE27" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF27" s="24"/>
+      <c r="AF27" s="16"/>
+      <c r="AG27" s="16"/>
+      <c r="AH27" s="16"/>
+      <c r="AI27" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ27" s="24"/>
     </row>
-    <row r="28" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="13">
         <v>21</v>
       </c>
       <c r="C28" s="14"/>
       <c r="D28" s="14"/>
       <c r="E28" s="22"/>
-      <c r="F28" s="46"/>
+      <c r="F28" s="26"/>
       <c r="G28" s="15"/>
       <c r="H28" s="17"/>
       <c r="I28" s="20">
@@ -9391,38 +9520,42 @@
         <v>0</v>
       </c>
       <c r="P28" s="16"/>
-      <c r="Q28" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R28" s="24"/>
-      <c r="S28" s="22"/>
-      <c r="T28" s="46"/>
-      <c r="U28" s="15"/>
-      <c r="V28" s="17"/>
-      <c r="W28" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X28" s="16"/>
-      <c r="Y28" s="16"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
+      <c r="S28" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T28" s="24"/>
+      <c r="U28" s="22"/>
+      <c r="V28" s="26"/>
+      <c r="W28" s="15"/>
+      <c r="X28" s="17"/>
+      <c r="Y28" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z28" s="16"/>
       <c r="AA28" s="16"/>
       <c r="AB28" s="16"/>
-      <c r="AC28" s="18">
+      <c r="AC28" s="16"/>
+      <c r="AD28" s="16"/>
+      <c r="AE28" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD28" s="16"/>
-      <c r="AE28" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF28" s="24"/>
+      <c r="AF28" s="16"/>
+      <c r="AG28" s="16"/>
+      <c r="AH28" s="16"/>
+      <c r="AI28" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ28" s="24"/>
     </row>
-    <row r="29" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="13"/>
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
       <c r="E29" s="22"/>
-      <c r="F29" s="46"/>
+      <c r="F29" s="26"/>
       <c r="G29" s="15"/>
       <c r="H29" s="17"/>
       <c r="I29" s="20">
@@ -9438,40 +9571,44 @@
         <v>0</v>
       </c>
       <c r="P29" s="16"/>
-      <c r="Q29" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R29" s="24"/>
-      <c r="S29" s="22"/>
-      <c r="T29" s="46"/>
-      <c r="U29" s="15"/>
-      <c r="V29" s="17"/>
-      <c r="W29" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X29" s="16"/>
-      <c r="Y29" s="16"/>
+      <c r="Q29" s="16"/>
+      <c r="R29" s="16"/>
+      <c r="S29" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T29" s="24"/>
+      <c r="U29" s="22"/>
+      <c r="V29" s="26"/>
+      <c r="W29" s="15"/>
+      <c r="X29" s="17"/>
+      <c r="Y29" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z29" s="16"/>
       <c r="AA29" s="16"/>
       <c r="AB29" s="16"/>
-      <c r="AC29" s="18">
+      <c r="AC29" s="16"/>
+      <c r="AD29" s="16"/>
+      <c r="AE29" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD29" s="16"/>
-      <c r="AE29" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF29" s="24"/>
+      <c r="AF29" s="16"/>
+      <c r="AG29" s="16"/>
+      <c r="AH29" s="16"/>
+      <c r="AI29" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ29" s="24"/>
     </row>
-    <row r="30" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="13">
         <v>22</v>
       </c>
       <c r="C30" s="14"/>
       <c r="D30" s="14"/>
       <c r="E30" s="22"/>
-      <c r="F30" s="46"/>
+      <c r="F30" s="26"/>
       <c r="G30" s="15"/>
       <c r="H30" s="17"/>
       <c r="I30" s="20">
@@ -9487,40 +9624,44 @@
         <v>0</v>
       </c>
       <c r="P30" s="16"/>
-      <c r="Q30" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R30" s="24"/>
-      <c r="S30" s="22"/>
-      <c r="T30" s="46"/>
-      <c r="U30" s="15"/>
-      <c r="V30" s="17"/>
-      <c r="W30" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X30" s="16"/>
-      <c r="Y30" s="16"/>
+      <c r="Q30" s="16"/>
+      <c r="R30" s="16"/>
+      <c r="S30" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T30" s="24"/>
+      <c r="U30" s="22"/>
+      <c r="V30" s="26"/>
+      <c r="W30" s="15"/>
+      <c r="X30" s="17"/>
+      <c r="Y30" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z30" s="16"/>
       <c r="AA30" s="16"/>
       <c r="AB30" s="16"/>
-      <c r="AC30" s="18">
+      <c r="AC30" s="16"/>
+      <c r="AD30" s="16"/>
+      <c r="AE30" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD30" s="16"/>
-      <c r="AE30" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF30" s="24"/>
+      <c r="AF30" s="16"/>
+      <c r="AG30" s="16"/>
+      <c r="AH30" s="16"/>
+      <c r="AI30" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ30" s="24"/>
     </row>
-    <row r="31" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="13">
         <v>23</v>
       </c>
       <c r="C31" s="14"/>
       <c r="D31" s="14"/>
       <c r="E31" s="22"/>
-      <c r="F31" s="46"/>
+      <c r="F31" s="26"/>
       <c r="G31" s="15"/>
       <c r="H31" s="17"/>
       <c r="I31" s="20">
@@ -9536,40 +9677,44 @@
         <v>0</v>
       </c>
       <c r="P31" s="16"/>
-      <c r="Q31" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R31" s="24"/>
-      <c r="S31" s="22"/>
-      <c r="T31" s="46"/>
-      <c r="U31" s="15"/>
-      <c r="V31" s="17"/>
-      <c r="W31" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X31" s="16"/>
-      <c r="Y31" s="16"/>
+      <c r="Q31" s="16"/>
+      <c r="R31" s="16"/>
+      <c r="S31" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T31" s="24"/>
+      <c r="U31" s="22"/>
+      <c r="V31" s="26"/>
+      <c r="W31" s="15"/>
+      <c r="X31" s="17"/>
+      <c r="Y31" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z31" s="16"/>
       <c r="AA31" s="16"/>
       <c r="AB31" s="16"/>
-      <c r="AC31" s="18">
+      <c r="AC31" s="16"/>
+      <c r="AD31" s="16"/>
+      <c r="AE31" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD31" s="16"/>
-      <c r="AE31" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF31" s="24"/>
+      <c r="AF31" s="16"/>
+      <c r="AG31" s="16"/>
+      <c r="AH31" s="16"/>
+      <c r="AI31" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ31" s="24"/>
     </row>
-    <row r="32" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="13">
         <v>24</v>
       </c>
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
       <c r="E32" s="22"/>
-      <c r="F32" s="46"/>
+      <c r="F32" s="26"/>
       <c r="G32" s="15"/>
       <c r="H32" s="17"/>
       <c r="I32" s="20">
@@ -9585,40 +9730,44 @@
         <v>0</v>
       </c>
       <c r="P32" s="16"/>
-      <c r="Q32" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R32" s="24"/>
-      <c r="S32" s="22"/>
-      <c r="T32" s="46"/>
-      <c r="U32" s="15"/>
-      <c r="V32" s="17"/>
-      <c r="W32" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X32" s="16"/>
-      <c r="Y32" s="16"/>
+      <c r="Q32" s="16"/>
+      <c r="R32" s="16"/>
+      <c r="S32" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T32" s="24"/>
+      <c r="U32" s="22"/>
+      <c r="V32" s="26"/>
+      <c r="W32" s="15"/>
+      <c r="X32" s="17"/>
+      <c r="Y32" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z32" s="16"/>
       <c r="AA32" s="16"/>
       <c r="AB32" s="16"/>
-      <c r="AC32" s="18">
+      <c r="AC32" s="16"/>
+      <c r="AD32" s="16"/>
+      <c r="AE32" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD32" s="16"/>
-      <c r="AE32" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF32" s="24"/>
+      <c r="AF32" s="16"/>
+      <c r="AG32" s="16"/>
+      <c r="AH32" s="16"/>
+      <c r="AI32" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ32" s="24"/>
     </row>
-    <row r="33" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="13">
         <v>25</v>
       </c>
       <c r="C33" s="14"/>
       <c r="D33" s="14"/>
       <c r="E33" s="22"/>
-      <c r="F33" s="46"/>
+      <c r="F33" s="26"/>
       <c r="G33" s="15"/>
       <c r="H33" s="17"/>
       <c r="I33" s="20">
@@ -9634,40 +9783,44 @@
         <v>0</v>
       </c>
       <c r="P33" s="16"/>
-      <c r="Q33" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R33" s="24"/>
-      <c r="S33" s="22"/>
-      <c r="T33" s="46"/>
-      <c r="U33" s="15"/>
-      <c r="V33" s="17"/>
-      <c r="W33" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X33" s="16"/>
-      <c r="Y33" s="16"/>
+      <c r="Q33" s="16"/>
+      <c r="R33" s="16"/>
+      <c r="S33" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T33" s="24"/>
+      <c r="U33" s="22"/>
+      <c r="V33" s="26"/>
+      <c r="W33" s="15"/>
+      <c r="X33" s="17"/>
+      <c r="Y33" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z33" s="16"/>
       <c r="AA33" s="16"/>
       <c r="AB33" s="16"/>
-      <c r="AC33" s="18">
+      <c r="AC33" s="16"/>
+      <c r="AD33" s="16"/>
+      <c r="AE33" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD33" s="16"/>
-      <c r="AE33" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF33" s="24"/>
+      <c r="AF33" s="16"/>
+      <c r="AG33" s="16"/>
+      <c r="AH33" s="16"/>
+      <c r="AI33" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ33" s="24"/>
     </row>
-    <row r="34" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="13">
         <v>26</v>
       </c>
       <c r="C34" s="14"/>
       <c r="D34" s="14"/>
       <c r="E34" s="22"/>
-      <c r="F34" s="46"/>
+      <c r="F34" s="26"/>
       <c r="G34" s="15"/>
       <c r="H34" s="17"/>
       <c r="I34" s="20">
@@ -9683,40 +9836,44 @@
         <v>0</v>
       </c>
       <c r="P34" s="16"/>
-      <c r="Q34" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R34" s="24"/>
-      <c r="S34" s="22"/>
-      <c r="T34" s="46"/>
-      <c r="U34" s="15"/>
-      <c r="V34" s="17"/>
-      <c r="W34" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X34" s="16"/>
-      <c r="Y34" s="16"/>
+      <c r="Q34" s="16"/>
+      <c r="R34" s="16"/>
+      <c r="S34" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T34" s="24"/>
+      <c r="U34" s="22"/>
+      <c r="V34" s="26"/>
+      <c r="W34" s="15"/>
+      <c r="X34" s="17"/>
+      <c r="Y34" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z34" s="16"/>
       <c r="AA34" s="16"/>
       <c r="AB34" s="16"/>
-      <c r="AC34" s="18">
+      <c r="AC34" s="16"/>
+      <c r="AD34" s="16"/>
+      <c r="AE34" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD34" s="16"/>
-      <c r="AE34" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF34" s="24"/>
+      <c r="AF34" s="16"/>
+      <c r="AG34" s="16"/>
+      <c r="AH34" s="16"/>
+      <c r="AI34" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ34" s="24"/>
     </row>
-    <row r="35" spans="2:32" s="12" customFormat="1" ht="126.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:36" s="12" customFormat="1" ht="126.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="13">
         <v>27</v>
       </c>
       <c r="C35" s="14"/>
       <c r="D35" s="14"/>
       <c r="E35" s="22"/>
-      <c r="F35" s="46"/>
+      <c r="F35" s="26"/>
       <c r="G35" s="15"/>
       <c r="H35" s="17"/>
       <c r="I35" s="20">
@@ -9732,40 +9889,44 @@
         <v>0</v>
       </c>
       <c r="P35" s="16"/>
-      <c r="Q35" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R35" s="24"/>
-      <c r="S35" s="22"/>
-      <c r="T35" s="46"/>
-      <c r="U35" s="15"/>
-      <c r="V35" s="17"/>
-      <c r="W35" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X35" s="16"/>
-      <c r="Y35" s="16"/>
+      <c r="Q35" s="16"/>
+      <c r="R35" s="16"/>
+      <c r="S35" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T35" s="24"/>
+      <c r="U35" s="22"/>
+      <c r="V35" s="26"/>
+      <c r="W35" s="15"/>
+      <c r="X35" s="17"/>
+      <c r="Y35" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z35" s="16"/>
       <c r="AA35" s="16"/>
       <c r="AB35" s="16"/>
-      <c r="AC35" s="18">
+      <c r="AC35" s="16"/>
+      <c r="AD35" s="16"/>
+      <c r="AE35" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD35" s="16"/>
-      <c r="AE35" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF35" s="24"/>
+      <c r="AF35" s="16"/>
+      <c r="AG35" s="16"/>
+      <c r="AH35" s="16"/>
+      <c r="AI35" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ35" s="24"/>
     </row>
-    <row r="36" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="13">
         <v>28</v>
       </c>
       <c r="C36" s="14"/>
       <c r="D36" s="14"/>
       <c r="E36" s="22"/>
-      <c r="F36" s="46"/>
+      <c r="F36" s="26"/>
       <c r="G36" s="15"/>
       <c r="H36" s="17"/>
       <c r="I36" s="20">
@@ -9781,40 +9942,44 @@
         <v>0</v>
       </c>
       <c r="P36" s="16"/>
-      <c r="Q36" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R36" s="24"/>
-      <c r="S36" s="22"/>
-      <c r="T36" s="46"/>
-      <c r="U36" s="15"/>
-      <c r="V36" s="17"/>
-      <c r="W36" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X36" s="16"/>
-      <c r="Y36" s="16"/>
+      <c r="Q36" s="16"/>
+      <c r="R36" s="16"/>
+      <c r="S36" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T36" s="24"/>
+      <c r="U36" s="22"/>
+      <c r="V36" s="26"/>
+      <c r="W36" s="15"/>
+      <c r="X36" s="17"/>
+      <c r="Y36" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z36" s="16"/>
       <c r="AA36" s="16"/>
       <c r="AB36" s="16"/>
-      <c r="AC36" s="18">
+      <c r="AC36" s="16"/>
+      <c r="AD36" s="16"/>
+      <c r="AE36" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD36" s="16"/>
-      <c r="AE36" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF36" s="24"/>
+      <c r="AF36" s="16"/>
+      <c r="AG36" s="16"/>
+      <c r="AH36" s="16"/>
+      <c r="AI36" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ36" s="24"/>
     </row>
-    <row r="37" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="13">
         <v>29</v>
       </c>
       <c r="C37" s="14"/>
       <c r="D37" s="14"/>
       <c r="E37" s="22"/>
-      <c r="F37" s="46"/>
+      <c r="F37" s="26"/>
       <c r="G37" s="15"/>
       <c r="H37" s="17"/>
       <c r="I37" s="20">
@@ -9830,40 +9995,44 @@
         <v>0</v>
       </c>
       <c r="P37" s="16"/>
-      <c r="Q37" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R37" s="24"/>
-      <c r="S37" s="22"/>
-      <c r="T37" s="46"/>
-      <c r="U37" s="15"/>
-      <c r="V37" s="17"/>
-      <c r="W37" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X37" s="16"/>
-      <c r="Y37" s="16"/>
+      <c r="Q37" s="16"/>
+      <c r="R37" s="16"/>
+      <c r="S37" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T37" s="24"/>
+      <c r="U37" s="22"/>
+      <c r="V37" s="26"/>
+      <c r="W37" s="15"/>
+      <c r="X37" s="17"/>
+      <c r="Y37" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z37" s="16"/>
       <c r="AA37" s="16"/>
       <c r="AB37" s="16"/>
-      <c r="AC37" s="18">
+      <c r="AC37" s="16"/>
+      <c r="AD37" s="16"/>
+      <c r="AE37" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD37" s="16"/>
-      <c r="AE37" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF37" s="24"/>
+      <c r="AF37" s="16"/>
+      <c r="AG37" s="16"/>
+      <c r="AH37" s="16"/>
+      <c r="AI37" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ37" s="24"/>
     </row>
-    <row r="38" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="13">
         <v>30</v>
       </c>
       <c r="C38" s="14"/>
       <c r="D38" s="14"/>
       <c r="E38" s="22"/>
-      <c r="F38" s="46"/>
+      <c r="F38" s="26"/>
       <c r="G38" s="15"/>
       <c r="H38" s="17"/>
       <c r="I38" s="20">
@@ -9879,40 +10048,44 @@
         <v>0</v>
       </c>
       <c r="P38" s="16"/>
-      <c r="Q38" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R38" s="24"/>
-      <c r="S38" s="22"/>
-      <c r="T38" s="46"/>
-      <c r="U38" s="15"/>
-      <c r="V38" s="17"/>
-      <c r="W38" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X38" s="16"/>
-      <c r="Y38" s="16"/>
+      <c r="Q38" s="16"/>
+      <c r="R38" s="16"/>
+      <c r="S38" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T38" s="24"/>
+      <c r="U38" s="22"/>
+      <c r="V38" s="26"/>
+      <c r="W38" s="15"/>
+      <c r="X38" s="17"/>
+      <c r="Y38" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z38" s="16"/>
       <c r="AA38" s="16"/>
       <c r="AB38" s="16"/>
-      <c r="AC38" s="18">
+      <c r="AC38" s="16"/>
+      <c r="AD38" s="16"/>
+      <c r="AE38" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD38" s="16"/>
-      <c r="AE38" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF38" s="24"/>
+      <c r="AF38" s="16"/>
+      <c r="AG38" s="16"/>
+      <c r="AH38" s="16"/>
+      <c r="AI38" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ38" s="24"/>
     </row>
-    <row r="39" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="13">
         <v>31</v>
       </c>
       <c r="C39" s="14"/>
       <c r="D39" s="14"/>
       <c r="E39" s="22"/>
-      <c r="F39" s="46"/>
+      <c r="F39" s="26"/>
       <c r="G39" s="15"/>
       <c r="H39" s="17"/>
       <c r="I39" s="20">
@@ -9928,40 +10101,44 @@
         <v>0</v>
       </c>
       <c r="P39" s="16"/>
-      <c r="Q39" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R39" s="24"/>
-      <c r="S39" s="22"/>
-      <c r="T39" s="46"/>
-      <c r="U39" s="15"/>
-      <c r="V39" s="17"/>
-      <c r="W39" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X39" s="16"/>
-      <c r="Y39" s="16"/>
+      <c r="Q39" s="16"/>
+      <c r="R39" s="16"/>
+      <c r="S39" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T39" s="24"/>
+      <c r="U39" s="22"/>
+      <c r="V39" s="26"/>
+      <c r="W39" s="15"/>
+      <c r="X39" s="17"/>
+      <c r="Y39" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z39" s="16"/>
       <c r="AA39" s="16"/>
       <c r="AB39" s="16"/>
-      <c r="AC39" s="18">
+      <c r="AC39" s="16"/>
+      <c r="AD39" s="16"/>
+      <c r="AE39" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD39" s="16"/>
-      <c r="AE39" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF39" s="24"/>
+      <c r="AF39" s="16"/>
+      <c r="AG39" s="16"/>
+      <c r="AH39" s="16"/>
+      <c r="AI39" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ39" s="24"/>
     </row>
-    <row r="40" spans="2:32" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:36" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="13">
         <v>32</v>
       </c>
       <c r="C40" s="14"/>
       <c r="D40" s="14"/>
       <c r="E40" s="22"/>
-      <c r="F40" s="46"/>
+      <c r="F40" s="26"/>
       <c r="G40" s="15"/>
       <c r="H40" s="17"/>
       <c r="I40" s="20">
@@ -9977,40 +10154,44 @@
         <v>0</v>
       </c>
       <c r="P40" s="16"/>
-      <c r="Q40" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R40" s="24"/>
-      <c r="S40" s="22"/>
-      <c r="T40" s="46"/>
-      <c r="U40" s="15"/>
-      <c r="V40" s="17"/>
-      <c r="W40" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X40" s="16"/>
-      <c r="Y40" s="16"/>
+      <c r="Q40" s="16"/>
+      <c r="R40" s="16"/>
+      <c r="S40" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T40" s="24"/>
+      <c r="U40" s="22"/>
+      <c r="V40" s="26"/>
+      <c r="W40" s="15"/>
+      <c r="X40" s="17"/>
+      <c r="Y40" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z40" s="16"/>
       <c r="AA40" s="16"/>
       <c r="AB40" s="16"/>
-      <c r="AC40" s="18">
+      <c r="AC40" s="16"/>
+      <c r="AD40" s="16"/>
+      <c r="AE40" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD40" s="16"/>
-      <c r="AE40" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF40" s="24"/>
+      <c r="AF40" s="16"/>
+      <c r="AG40" s="16"/>
+      <c r="AH40" s="16"/>
+      <c r="AI40" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ40" s="24"/>
     </row>
-    <row r="41" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="13">
         <v>33</v>
       </c>
       <c r="C41" s="14"/>
       <c r="D41" s="14"/>
       <c r="E41" s="22"/>
-      <c r="F41" s="46"/>
+      <c r="F41" s="26"/>
       <c r="G41" s="15"/>
       <c r="H41" s="17"/>
       <c r="I41" s="20">
@@ -10026,40 +10207,44 @@
         <v>0</v>
       </c>
       <c r="P41" s="16"/>
-      <c r="Q41" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R41" s="24"/>
-      <c r="S41" s="22"/>
-      <c r="T41" s="46"/>
-      <c r="U41" s="15"/>
-      <c r="V41" s="17"/>
-      <c r="W41" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X41" s="16"/>
-      <c r="Y41" s="16"/>
+      <c r="Q41" s="16"/>
+      <c r="R41" s="16"/>
+      <c r="S41" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T41" s="24"/>
+      <c r="U41" s="22"/>
+      <c r="V41" s="26"/>
+      <c r="W41" s="15"/>
+      <c r="X41" s="17"/>
+      <c r="Y41" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z41" s="16"/>
       <c r="AA41" s="16"/>
       <c r="AB41" s="16"/>
-      <c r="AC41" s="18">
+      <c r="AC41" s="16"/>
+      <c r="AD41" s="16"/>
+      <c r="AE41" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD41" s="16"/>
-      <c r="AE41" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF41" s="24"/>
+      <c r="AF41" s="16"/>
+      <c r="AG41" s="16"/>
+      <c r="AH41" s="16"/>
+      <c r="AI41" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ41" s="24"/>
     </row>
-    <row r="42" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="13">
         <v>34</v>
       </c>
       <c r="C42" s="14"/>
       <c r="D42" s="14"/>
       <c r="E42" s="22"/>
-      <c r="F42" s="46"/>
+      <c r="F42" s="26"/>
       <c r="G42" s="15"/>
       <c r="H42" s="17"/>
       <c r="I42" s="20">
@@ -10075,40 +10260,44 @@
         <v>0</v>
       </c>
       <c r="P42" s="16"/>
-      <c r="Q42" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R42" s="24"/>
-      <c r="S42" s="22"/>
-      <c r="T42" s="46"/>
-      <c r="U42" s="15"/>
-      <c r="V42" s="17"/>
-      <c r="W42" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X42" s="16"/>
-      <c r="Y42" s="16"/>
+      <c r="Q42" s="16"/>
+      <c r="R42" s="16"/>
+      <c r="S42" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T42" s="24"/>
+      <c r="U42" s="22"/>
+      <c r="V42" s="26"/>
+      <c r="W42" s="15"/>
+      <c r="X42" s="17"/>
+      <c r="Y42" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z42" s="16"/>
       <c r="AA42" s="16"/>
       <c r="AB42" s="16"/>
-      <c r="AC42" s="18">
+      <c r="AC42" s="16"/>
+      <c r="AD42" s="16"/>
+      <c r="AE42" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD42" s="16"/>
-      <c r="AE42" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF42" s="24"/>
+      <c r="AF42" s="16"/>
+      <c r="AG42" s="16"/>
+      <c r="AH42" s="16"/>
+      <c r="AI42" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ42" s="24"/>
     </row>
-    <row r="43" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="13">
         <v>35</v>
       </c>
       <c r="C43" s="14"/>
       <c r="D43" s="14"/>
       <c r="E43" s="22"/>
-      <c r="F43" s="46"/>
+      <c r="F43" s="26"/>
       <c r="G43" s="15"/>
       <c r="H43" s="17"/>
       <c r="I43" s="20">
@@ -10124,40 +10313,44 @@
         <v>0</v>
       </c>
       <c r="P43" s="16"/>
-      <c r="Q43" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R43" s="24"/>
-      <c r="S43" s="22"/>
-      <c r="T43" s="46"/>
-      <c r="U43" s="15"/>
-      <c r="V43" s="17"/>
-      <c r="W43" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X43" s="16"/>
-      <c r="Y43" s="16"/>
+      <c r="Q43" s="16"/>
+      <c r="R43" s="16"/>
+      <c r="S43" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T43" s="24"/>
+      <c r="U43" s="22"/>
+      <c r="V43" s="26"/>
+      <c r="W43" s="15"/>
+      <c r="X43" s="17"/>
+      <c r="Y43" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z43" s="16"/>
       <c r="AA43" s="16"/>
       <c r="AB43" s="16"/>
-      <c r="AC43" s="18">
+      <c r="AC43" s="16"/>
+      <c r="AD43" s="16"/>
+      <c r="AE43" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD43" s="16"/>
-      <c r="AE43" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF43" s="24"/>
+      <c r="AF43" s="16"/>
+      <c r="AG43" s="16"/>
+      <c r="AH43" s="16"/>
+      <c r="AI43" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ43" s="24"/>
     </row>
-    <row r="44" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="13">
         <v>36</v>
       </c>
       <c r="C44" s="14"/>
       <c r="D44" s="14"/>
       <c r="E44" s="22"/>
-      <c r="F44" s="46"/>
+      <c r="F44" s="26"/>
       <c r="G44" s="15"/>
       <c r="H44" s="17"/>
       <c r="I44" s="20">
@@ -10173,40 +10366,44 @@
         <v>0</v>
       </c>
       <c r="P44" s="16"/>
-      <c r="Q44" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R44" s="24"/>
-      <c r="S44" s="22"/>
-      <c r="T44" s="46"/>
-      <c r="U44" s="15"/>
-      <c r="V44" s="17"/>
-      <c r="W44" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X44" s="16"/>
-      <c r="Y44" s="16"/>
+      <c r="Q44" s="16"/>
+      <c r="R44" s="16"/>
+      <c r="S44" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T44" s="24"/>
+      <c r="U44" s="22"/>
+      <c r="V44" s="26"/>
+      <c r="W44" s="15"/>
+      <c r="X44" s="17"/>
+      <c r="Y44" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z44" s="16"/>
       <c r="AA44" s="16"/>
       <c r="AB44" s="16"/>
-      <c r="AC44" s="18">
+      <c r="AC44" s="16"/>
+      <c r="AD44" s="16"/>
+      <c r="AE44" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD44" s="16"/>
-      <c r="AE44" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF44" s="24"/>
+      <c r="AF44" s="16"/>
+      <c r="AG44" s="16"/>
+      <c r="AH44" s="16"/>
+      <c r="AI44" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ44" s="24"/>
     </row>
-    <row r="45" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="13">
         <v>37</v>
       </c>
       <c r="C45" s="14"/>
       <c r="D45" s="14"/>
       <c r="E45" s="22"/>
-      <c r="F45" s="46"/>
+      <c r="F45" s="26"/>
       <c r="G45" s="15"/>
       <c r="H45" s="17"/>
       <c r="I45" s="20">
@@ -10222,40 +10419,44 @@
         <v>0</v>
       </c>
       <c r="P45" s="16"/>
-      <c r="Q45" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R45" s="24"/>
-      <c r="S45" s="22"/>
-      <c r="T45" s="46"/>
-      <c r="U45" s="15"/>
-      <c r="V45" s="17"/>
-      <c r="W45" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X45" s="16"/>
-      <c r="Y45" s="16"/>
+      <c r="Q45" s="16"/>
+      <c r="R45" s="16"/>
+      <c r="S45" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T45" s="24"/>
+      <c r="U45" s="22"/>
+      <c r="V45" s="26"/>
+      <c r="W45" s="15"/>
+      <c r="X45" s="17"/>
+      <c r="Y45" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z45" s="16"/>
       <c r="AA45" s="16"/>
       <c r="AB45" s="16"/>
-      <c r="AC45" s="18">
+      <c r="AC45" s="16"/>
+      <c r="AD45" s="16"/>
+      <c r="AE45" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD45" s="16"/>
-      <c r="AE45" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF45" s="24"/>
+      <c r="AF45" s="16"/>
+      <c r="AG45" s="16"/>
+      <c r="AH45" s="16"/>
+      <c r="AI45" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ45" s="24"/>
     </row>
-    <row r="46" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="13">
         <v>38</v>
       </c>
       <c r="C46" s="14"/>
       <c r="D46" s="14"/>
       <c r="E46" s="22"/>
-      <c r="F46" s="46"/>
+      <c r="F46" s="26"/>
       <c r="G46" s="15"/>
       <c r="H46" s="17"/>
       <c r="I46" s="20">
@@ -10271,40 +10472,44 @@
         <v>0</v>
       </c>
       <c r="P46" s="16"/>
-      <c r="Q46" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R46" s="24"/>
-      <c r="S46" s="22"/>
-      <c r="T46" s="46"/>
-      <c r="U46" s="15"/>
-      <c r="V46" s="17"/>
-      <c r="W46" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X46" s="16"/>
-      <c r="Y46" s="16"/>
+      <c r="Q46" s="16"/>
+      <c r="R46" s="16"/>
+      <c r="S46" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T46" s="24"/>
+      <c r="U46" s="22"/>
+      <c r="V46" s="26"/>
+      <c r="W46" s="15"/>
+      <c r="X46" s="17"/>
+      <c r="Y46" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z46" s="16"/>
       <c r="AA46" s="16"/>
       <c r="AB46" s="16"/>
-      <c r="AC46" s="18">
+      <c r="AC46" s="16"/>
+      <c r="AD46" s="16"/>
+      <c r="AE46" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD46" s="16"/>
-      <c r="AE46" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF46" s="24"/>
+      <c r="AF46" s="16"/>
+      <c r="AG46" s="16"/>
+      <c r="AH46" s="16"/>
+      <c r="AI46" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ46" s="24"/>
     </row>
-    <row r="47" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="13">
         <v>39</v>
       </c>
       <c r="C47" s="14"/>
       <c r="D47" s="14"/>
       <c r="E47" s="22"/>
-      <c r="F47" s="46"/>
+      <c r="F47" s="26"/>
       <c r="G47" s="15"/>
       <c r="H47" s="17"/>
       <c r="I47" s="20">
@@ -10320,40 +10525,44 @@
         <v>0</v>
       </c>
       <c r="P47" s="16"/>
-      <c r="Q47" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R47" s="24"/>
-      <c r="S47" s="22"/>
-      <c r="T47" s="46"/>
-      <c r="U47" s="15"/>
-      <c r="V47" s="17"/>
-      <c r="W47" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X47" s="16"/>
-      <c r="Y47" s="16"/>
+      <c r="Q47" s="16"/>
+      <c r="R47" s="16"/>
+      <c r="S47" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T47" s="24"/>
+      <c r="U47" s="22"/>
+      <c r="V47" s="26"/>
+      <c r="W47" s="15"/>
+      <c r="X47" s="17"/>
+      <c r="Y47" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z47" s="16"/>
       <c r="AA47" s="16"/>
       <c r="AB47" s="16"/>
-      <c r="AC47" s="18">
+      <c r="AC47" s="16"/>
+      <c r="AD47" s="16"/>
+      <c r="AE47" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD47" s="16"/>
-      <c r="AE47" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF47" s="24"/>
+      <c r="AF47" s="16"/>
+      <c r="AG47" s="16"/>
+      <c r="AH47" s="16"/>
+      <c r="AI47" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ47" s="24"/>
     </row>
-    <row r="48" spans="2:32" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:36" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="13">
         <v>40</v>
       </c>
       <c r="C48" s="14"/>
       <c r="D48" s="14"/>
       <c r="E48" s="22"/>
-      <c r="F48" s="46"/>
+      <c r="F48" s="26"/>
       <c r="G48" s="15"/>
       <c r="H48" s="17"/>
       <c r="I48" s="20">
@@ -10369,40 +10578,44 @@
         <v>0</v>
       </c>
       <c r="P48" s="16"/>
-      <c r="Q48" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R48" s="24"/>
-      <c r="S48" s="22"/>
-      <c r="T48" s="46"/>
-      <c r="U48" s="15"/>
-      <c r="V48" s="17"/>
-      <c r="W48" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X48" s="16"/>
-      <c r="Y48" s="16"/>
+      <c r="Q48" s="16"/>
+      <c r="R48" s="16"/>
+      <c r="S48" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T48" s="24"/>
+      <c r="U48" s="22"/>
+      <c r="V48" s="26"/>
+      <c r="W48" s="15"/>
+      <c r="X48" s="17"/>
+      <c r="Y48" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z48" s="16"/>
       <c r="AA48" s="16"/>
       <c r="AB48" s="16"/>
-      <c r="AC48" s="18">
+      <c r="AC48" s="16"/>
+      <c r="AD48" s="16"/>
+      <c r="AE48" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD48" s="16"/>
-      <c r="AE48" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF48" s="24"/>
+      <c r="AF48" s="16"/>
+      <c r="AG48" s="16"/>
+      <c r="AH48" s="16"/>
+      <c r="AI48" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ48" s="24"/>
     </row>
-    <row r="49" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="13">
         <v>41</v>
       </c>
       <c r="C49" s="14"/>
       <c r="D49" s="14"/>
       <c r="E49" s="22"/>
-      <c r="F49" s="46"/>
+      <c r="F49" s="26"/>
       <c r="G49" s="15"/>
       <c r="H49" s="17"/>
       <c r="I49" s="20">
@@ -10418,40 +10631,44 @@
         <v>0</v>
       </c>
       <c r="P49" s="16"/>
-      <c r="Q49" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R49" s="24"/>
-      <c r="S49" s="22"/>
-      <c r="T49" s="46"/>
-      <c r="U49" s="15"/>
-      <c r="V49" s="17"/>
-      <c r="W49" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X49" s="16"/>
-      <c r="Y49" s="16"/>
+      <c r="Q49" s="16"/>
+      <c r="R49" s="16"/>
+      <c r="S49" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T49" s="24"/>
+      <c r="U49" s="22"/>
+      <c r="V49" s="26"/>
+      <c r="W49" s="15"/>
+      <c r="X49" s="17"/>
+      <c r="Y49" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z49" s="16"/>
       <c r="AA49" s="16"/>
       <c r="AB49" s="16"/>
-      <c r="AC49" s="18">
+      <c r="AC49" s="16"/>
+      <c r="AD49" s="16"/>
+      <c r="AE49" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD49" s="16"/>
-      <c r="AE49" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF49" s="24"/>
+      <c r="AF49" s="16"/>
+      <c r="AG49" s="16"/>
+      <c r="AH49" s="16"/>
+      <c r="AI49" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ49" s="24"/>
     </row>
-    <row r="50" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="13">
         <v>42</v>
       </c>
       <c r="C50" s="14"/>
       <c r="D50" s="14"/>
       <c r="E50" s="22"/>
-      <c r="F50" s="46"/>
+      <c r="F50" s="26"/>
       <c r="G50" s="15"/>
       <c r="H50" s="17"/>
       <c r="I50" s="20">
@@ -10467,40 +10684,44 @@
         <v>0</v>
       </c>
       <c r="P50" s="16"/>
-      <c r="Q50" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R50" s="24"/>
-      <c r="S50" s="22"/>
-      <c r="T50" s="46"/>
-      <c r="U50" s="15"/>
-      <c r="V50" s="17"/>
-      <c r="W50" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X50" s="16"/>
-      <c r="Y50" s="16"/>
+      <c r="Q50" s="16"/>
+      <c r="R50" s="16"/>
+      <c r="S50" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T50" s="24"/>
+      <c r="U50" s="22"/>
+      <c r="V50" s="26"/>
+      <c r="W50" s="15"/>
+      <c r="X50" s="17"/>
+      <c r="Y50" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z50" s="16"/>
       <c r="AA50" s="16"/>
       <c r="AB50" s="16"/>
-      <c r="AC50" s="18">
+      <c r="AC50" s="16"/>
+      <c r="AD50" s="16"/>
+      <c r="AE50" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD50" s="16"/>
-      <c r="AE50" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF50" s="24"/>
+      <c r="AF50" s="16"/>
+      <c r="AG50" s="16"/>
+      <c r="AH50" s="16"/>
+      <c r="AI50" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ50" s="24"/>
     </row>
-    <row r="51" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="13">
         <v>43</v>
       </c>
       <c r="C51" s="14"/>
       <c r="D51" s="14"/>
       <c r="E51" s="22"/>
-      <c r="F51" s="46"/>
+      <c r="F51" s="26"/>
       <c r="G51" s="15"/>
       <c r="H51" s="17"/>
       <c r="I51" s="20">
@@ -10516,40 +10737,44 @@
         <v>0</v>
       </c>
       <c r="P51" s="16"/>
-      <c r="Q51" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R51" s="24"/>
-      <c r="S51" s="22"/>
-      <c r="T51" s="46"/>
-      <c r="U51" s="15"/>
-      <c r="V51" s="17"/>
-      <c r="W51" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X51" s="16"/>
-      <c r="Y51" s="16"/>
+      <c r="Q51" s="16"/>
+      <c r="R51" s="16"/>
+      <c r="S51" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T51" s="24"/>
+      <c r="U51" s="22"/>
+      <c r="V51" s="26"/>
+      <c r="W51" s="15"/>
+      <c r="X51" s="17"/>
+      <c r="Y51" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z51" s="16"/>
       <c r="AA51" s="16"/>
       <c r="AB51" s="16"/>
-      <c r="AC51" s="18">
+      <c r="AC51" s="16"/>
+      <c r="AD51" s="16"/>
+      <c r="AE51" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD51" s="16"/>
-      <c r="AE51" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF51" s="24"/>
+      <c r="AF51" s="16"/>
+      <c r="AG51" s="16"/>
+      <c r="AH51" s="16"/>
+      <c r="AI51" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ51" s="24"/>
     </row>
-    <row r="52" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="13">
         <v>44</v>
       </c>
       <c r="C52" s="14"/>
       <c r="D52" s="14"/>
       <c r="E52" s="22"/>
-      <c r="F52" s="46"/>
+      <c r="F52" s="26"/>
       <c r="G52" s="15"/>
       <c r="H52" s="17"/>
       <c r="I52" s="20">
@@ -10565,40 +10790,44 @@
         <v>0</v>
       </c>
       <c r="P52" s="16"/>
-      <c r="Q52" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R52" s="24"/>
-      <c r="S52" s="22"/>
-      <c r="T52" s="46"/>
-      <c r="U52" s="15"/>
-      <c r="V52" s="17"/>
-      <c r="W52" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X52" s="16"/>
-      <c r="Y52" s="16"/>
+      <c r="Q52" s="16"/>
+      <c r="R52" s="16"/>
+      <c r="S52" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T52" s="24"/>
+      <c r="U52" s="22"/>
+      <c r="V52" s="26"/>
+      <c r="W52" s="15"/>
+      <c r="X52" s="17"/>
+      <c r="Y52" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z52" s="16"/>
       <c r="AA52" s="16"/>
       <c r="AB52" s="16"/>
-      <c r="AC52" s="18">
+      <c r="AC52" s="16"/>
+      <c r="AD52" s="16"/>
+      <c r="AE52" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD52" s="16"/>
-      <c r="AE52" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF52" s="24"/>
+      <c r="AF52" s="16"/>
+      <c r="AG52" s="16"/>
+      <c r="AH52" s="16"/>
+      <c r="AI52" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ52" s="24"/>
     </row>
-    <row r="53" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="13">
         <v>45</v>
       </c>
       <c r="C53" s="14"/>
       <c r="D53" s="14"/>
       <c r="E53" s="22"/>
-      <c r="F53" s="46"/>
+      <c r="F53" s="26"/>
       <c r="G53" s="15"/>
       <c r="H53" s="17"/>
       <c r="I53" s="20">
@@ -10614,40 +10843,44 @@
         <v>0</v>
       </c>
       <c r="P53" s="16"/>
-      <c r="Q53" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R53" s="24"/>
-      <c r="S53" s="22"/>
-      <c r="T53" s="46"/>
-      <c r="U53" s="15"/>
-      <c r="V53" s="17"/>
-      <c r="W53" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X53" s="16"/>
-      <c r="Y53" s="16"/>
+      <c r="Q53" s="16"/>
+      <c r="R53" s="16"/>
+      <c r="S53" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T53" s="24"/>
+      <c r="U53" s="22"/>
+      <c r="V53" s="26"/>
+      <c r="W53" s="15"/>
+      <c r="X53" s="17"/>
+      <c r="Y53" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z53" s="16"/>
       <c r="AA53" s="16"/>
       <c r="AB53" s="16"/>
-      <c r="AC53" s="18">
+      <c r="AC53" s="16"/>
+      <c r="AD53" s="16"/>
+      <c r="AE53" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD53" s="16"/>
-      <c r="AE53" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF53" s="24"/>
+      <c r="AF53" s="16"/>
+      <c r="AG53" s="16"/>
+      <c r="AH53" s="16"/>
+      <c r="AI53" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ53" s="24"/>
     </row>
-    <row r="54" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="13">
         <v>46</v>
       </c>
       <c r="C54" s="14"/>
       <c r="D54" s="14"/>
       <c r="E54" s="22"/>
-      <c r="F54" s="46"/>
+      <c r="F54" s="26"/>
       <c r="G54" s="15"/>
       <c r="H54" s="17"/>
       <c r="I54" s="20">
@@ -10663,40 +10896,44 @@
         <v>0</v>
       </c>
       <c r="P54" s="16"/>
-      <c r="Q54" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R54" s="24"/>
-      <c r="S54" s="22"/>
-      <c r="T54" s="46"/>
-      <c r="U54" s="15"/>
-      <c r="V54" s="17"/>
-      <c r="W54" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X54" s="16"/>
-      <c r="Y54" s="16"/>
+      <c r="Q54" s="16"/>
+      <c r="R54" s="16"/>
+      <c r="S54" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T54" s="24"/>
+      <c r="U54" s="22"/>
+      <c r="V54" s="26"/>
+      <c r="W54" s="15"/>
+      <c r="X54" s="17"/>
+      <c r="Y54" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z54" s="16"/>
       <c r="AA54" s="16"/>
       <c r="AB54" s="16"/>
-      <c r="AC54" s="18">
+      <c r="AC54" s="16"/>
+      <c r="AD54" s="16"/>
+      <c r="AE54" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD54" s="16"/>
-      <c r="AE54" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF54" s="24"/>
+      <c r="AF54" s="16"/>
+      <c r="AG54" s="16"/>
+      <c r="AH54" s="16"/>
+      <c r="AI54" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ54" s="24"/>
     </row>
-    <row r="55" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="13">
         <v>47</v>
       </c>
       <c r="C55" s="14"/>
       <c r="D55" s="14"/>
       <c r="E55" s="22"/>
-      <c r="F55" s="46"/>
+      <c r="F55" s="26"/>
       <c r="G55" s="15"/>
       <c r="H55" s="17"/>
       <c r="I55" s="20">
@@ -10712,40 +10949,44 @@
         <v>0</v>
       </c>
       <c r="P55" s="16"/>
-      <c r="Q55" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R55" s="24"/>
-      <c r="S55" s="22"/>
-      <c r="T55" s="46"/>
-      <c r="U55" s="15"/>
-      <c r="V55" s="17"/>
-      <c r="W55" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X55" s="16"/>
-      <c r="Y55" s="16"/>
+      <c r="Q55" s="16"/>
+      <c r="R55" s="16"/>
+      <c r="S55" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T55" s="24"/>
+      <c r="U55" s="22"/>
+      <c r="V55" s="26"/>
+      <c r="W55" s="15"/>
+      <c r="X55" s="17"/>
+      <c r="Y55" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z55" s="16"/>
       <c r="AA55" s="16"/>
       <c r="AB55" s="16"/>
-      <c r="AC55" s="18">
+      <c r="AC55" s="16"/>
+      <c r="AD55" s="16"/>
+      <c r="AE55" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD55" s="16"/>
-      <c r="AE55" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF55" s="24"/>
+      <c r="AF55" s="16"/>
+      <c r="AG55" s="16"/>
+      <c r="AH55" s="16"/>
+      <c r="AI55" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ55" s="24"/>
     </row>
-    <row r="56" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="13">
         <v>48</v>
       </c>
       <c r="C56" s="14"/>
       <c r="D56" s="14"/>
       <c r="E56" s="22"/>
-      <c r="F56" s="46"/>
+      <c r="F56" s="26"/>
       <c r="G56" s="15"/>
       <c r="H56" s="17"/>
       <c r="I56" s="20">
@@ -10761,40 +11002,44 @@
         <v>0</v>
       </c>
       <c r="P56" s="16"/>
-      <c r="Q56" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R56" s="24"/>
-      <c r="S56" s="22"/>
-      <c r="T56" s="46"/>
-      <c r="U56" s="15"/>
-      <c r="V56" s="17"/>
-      <c r="W56" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X56" s="16"/>
-      <c r="Y56" s="16"/>
+      <c r="Q56" s="16"/>
+      <c r="R56" s="16"/>
+      <c r="S56" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T56" s="24"/>
+      <c r="U56" s="22"/>
+      <c r="V56" s="26"/>
+      <c r="W56" s="15"/>
+      <c r="X56" s="17"/>
+      <c r="Y56" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z56" s="16"/>
       <c r="AA56" s="16"/>
       <c r="AB56" s="16"/>
-      <c r="AC56" s="18">
+      <c r="AC56" s="16"/>
+      <c r="AD56" s="16"/>
+      <c r="AE56" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD56" s="16"/>
-      <c r="AE56" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF56" s="24"/>
+      <c r="AF56" s="16"/>
+      <c r="AG56" s="16"/>
+      <c r="AH56" s="16"/>
+      <c r="AI56" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ56" s="24"/>
     </row>
-    <row r="57" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="13">
         <v>49</v>
       </c>
       <c r="C57" s="14"/>
       <c r="D57" s="14"/>
       <c r="E57" s="22"/>
-      <c r="F57" s="46"/>
+      <c r="F57" s="26"/>
       <c r="G57" s="15"/>
       <c r="H57" s="17"/>
       <c r="I57" s="20">
@@ -10810,40 +11055,44 @@
         <v>0</v>
       </c>
       <c r="P57" s="16"/>
-      <c r="Q57" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R57" s="24"/>
-      <c r="S57" s="22"/>
-      <c r="T57" s="46"/>
-      <c r="U57" s="15"/>
-      <c r="V57" s="17"/>
-      <c r="W57" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X57" s="16"/>
-      <c r="Y57" s="16"/>
+      <c r="Q57" s="16"/>
+      <c r="R57" s="16"/>
+      <c r="S57" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T57" s="24"/>
+      <c r="U57" s="22"/>
+      <c r="V57" s="26"/>
+      <c r="W57" s="15"/>
+      <c r="X57" s="17"/>
+      <c r="Y57" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z57" s="16"/>
       <c r="AA57" s="16"/>
       <c r="AB57" s="16"/>
-      <c r="AC57" s="18">
+      <c r="AC57" s="16"/>
+      <c r="AD57" s="16"/>
+      <c r="AE57" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD57" s="16"/>
-      <c r="AE57" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF57" s="24"/>
+      <c r="AF57" s="16"/>
+      <c r="AG57" s="16"/>
+      <c r="AH57" s="16"/>
+      <c r="AI57" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ57" s="24"/>
     </row>
-    <row r="58" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="13">
         <v>50</v>
       </c>
       <c r="C58" s="14"/>
       <c r="D58" s="14"/>
       <c r="E58" s="22"/>
-      <c r="F58" s="46"/>
+      <c r="F58" s="26"/>
       <c r="G58" s="15"/>
       <c r="H58" s="17"/>
       <c r="I58" s="20">
@@ -10859,40 +11108,44 @@
         <v>0</v>
       </c>
       <c r="P58" s="16"/>
-      <c r="Q58" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R58" s="24"/>
-      <c r="S58" s="22"/>
-      <c r="T58" s="46"/>
-      <c r="U58" s="15"/>
-      <c r="V58" s="17"/>
-      <c r="W58" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X58" s="16"/>
-      <c r="Y58" s="16"/>
+      <c r="Q58" s="16"/>
+      <c r="R58" s="16"/>
+      <c r="S58" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T58" s="24"/>
+      <c r="U58" s="22"/>
+      <c r="V58" s="26"/>
+      <c r="W58" s="15"/>
+      <c r="X58" s="17"/>
+      <c r="Y58" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z58" s="16"/>
       <c r="AA58" s="16"/>
       <c r="AB58" s="16"/>
-      <c r="AC58" s="18">
+      <c r="AC58" s="16"/>
+      <c r="AD58" s="16"/>
+      <c r="AE58" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD58" s="16"/>
-      <c r="AE58" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF58" s="24"/>
+      <c r="AF58" s="16"/>
+      <c r="AG58" s="16"/>
+      <c r="AH58" s="16"/>
+      <c r="AI58" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ58" s="24"/>
     </row>
-    <row r="59" spans="2:32" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:36" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="13">
         <v>51</v>
       </c>
       <c r="C59" s="14"/>
       <c r="D59" s="14"/>
       <c r="E59" s="22"/>
-      <c r="F59" s="46"/>
+      <c r="F59" s="26"/>
       <c r="G59" s="15"/>
       <c r="H59" s="17"/>
       <c r="I59" s="20">
@@ -10908,40 +11161,44 @@
         <v>0</v>
       </c>
       <c r="P59" s="16"/>
-      <c r="Q59" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R59" s="24"/>
-      <c r="S59" s="22"/>
-      <c r="T59" s="46"/>
-      <c r="U59" s="15"/>
-      <c r="V59" s="17"/>
-      <c r="W59" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X59" s="16"/>
-      <c r="Y59" s="16"/>
+      <c r="Q59" s="16"/>
+      <c r="R59" s="16"/>
+      <c r="S59" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T59" s="24"/>
+      <c r="U59" s="22"/>
+      <c r="V59" s="26"/>
+      <c r="W59" s="15"/>
+      <c r="X59" s="17"/>
+      <c r="Y59" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z59" s="16"/>
       <c r="AA59" s="16"/>
       <c r="AB59" s="16"/>
-      <c r="AC59" s="18">
+      <c r="AC59" s="16"/>
+      <c r="AD59" s="16"/>
+      <c r="AE59" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD59" s="16"/>
-      <c r="AE59" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF59" s="24"/>
+      <c r="AF59" s="16"/>
+      <c r="AG59" s="16"/>
+      <c r="AH59" s="16"/>
+      <c r="AI59" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ59" s="24"/>
     </row>
-    <row r="60" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="13">
         <v>52</v>
       </c>
       <c r="C60" s="14"/>
       <c r="D60" s="14"/>
       <c r="E60" s="22"/>
-      <c r="F60" s="46"/>
+      <c r="F60" s="26"/>
       <c r="G60" s="15"/>
       <c r="H60" s="17"/>
       <c r="I60" s="20">
@@ -10957,40 +11214,44 @@
         <v>0</v>
       </c>
       <c r="P60" s="16"/>
-      <c r="Q60" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R60" s="24"/>
-      <c r="S60" s="22"/>
-      <c r="T60" s="46"/>
-      <c r="U60" s="15"/>
-      <c r="V60" s="17"/>
-      <c r="W60" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X60" s="16"/>
-      <c r="Y60" s="16"/>
+      <c r="Q60" s="16"/>
+      <c r="R60" s="16"/>
+      <c r="S60" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T60" s="24"/>
+      <c r="U60" s="22"/>
+      <c r="V60" s="26"/>
+      <c r="W60" s="15"/>
+      <c r="X60" s="17"/>
+      <c r="Y60" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z60" s="16"/>
       <c r="AA60" s="16"/>
       <c r="AB60" s="16"/>
-      <c r="AC60" s="18">
+      <c r="AC60" s="16"/>
+      <c r="AD60" s="16"/>
+      <c r="AE60" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD60" s="16"/>
-      <c r="AE60" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF60" s="24"/>
+      <c r="AF60" s="16"/>
+      <c r="AG60" s="16"/>
+      <c r="AH60" s="16"/>
+      <c r="AI60" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ60" s="24"/>
     </row>
-    <row r="61" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="13">
         <v>53</v>
       </c>
       <c r="C61" s="14"/>
       <c r="D61" s="14"/>
       <c r="E61" s="22"/>
-      <c r="F61" s="46"/>
+      <c r="F61" s="26"/>
       <c r="G61" s="15"/>
       <c r="H61" s="17"/>
       <c r="I61" s="20">
@@ -11006,40 +11267,44 @@
         <v>0</v>
       </c>
       <c r="P61" s="16"/>
-      <c r="Q61" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R61" s="24"/>
-      <c r="S61" s="22"/>
-      <c r="T61" s="46"/>
-      <c r="U61" s="15"/>
-      <c r="V61" s="17"/>
-      <c r="W61" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X61" s="16"/>
-      <c r="Y61" s="16"/>
+      <c r="Q61" s="16"/>
+      <c r="R61" s="16"/>
+      <c r="S61" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T61" s="24"/>
+      <c r="U61" s="22"/>
+      <c r="V61" s="26"/>
+      <c r="W61" s="15"/>
+      <c r="X61" s="17"/>
+      <c r="Y61" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z61" s="16"/>
       <c r="AA61" s="16"/>
       <c r="AB61" s="16"/>
-      <c r="AC61" s="18">
+      <c r="AC61" s="16"/>
+      <c r="AD61" s="16"/>
+      <c r="AE61" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD61" s="16"/>
-      <c r="AE61" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF61" s="24"/>
+      <c r="AF61" s="16"/>
+      <c r="AG61" s="16"/>
+      <c r="AH61" s="16"/>
+      <c r="AI61" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ61" s="24"/>
     </row>
-    <row r="62" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="13">
         <v>54</v>
       </c>
       <c r="C62" s="14"/>
       <c r="D62" s="14"/>
       <c r="E62" s="22"/>
-      <c r="F62" s="46"/>
+      <c r="F62" s="26"/>
       <c r="G62" s="15"/>
       <c r="H62" s="17"/>
       <c r="I62" s="20">
@@ -11055,40 +11320,44 @@
         <v>0</v>
       </c>
       <c r="P62" s="16"/>
-      <c r="Q62" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R62" s="24"/>
-      <c r="S62" s="22"/>
-      <c r="T62" s="46"/>
-      <c r="U62" s="15"/>
-      <c r="V62" s="17"/>
-      <c r="W62" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X62" s="16"/>
-      <c r="Y62" s="16"/>
+      <c r="Q62" s="16"/>
+      <c r="R62" s="16"/>
+      <c r="S62" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T62" s="24"/>
+      <c r="U62" s="22"/>
+      <c r="V62" s="26"/>
+      <c r="W62" s="15"/>
+      <c r="X62" s="17"/>
+      <c r="Y62" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z62" s="16"/>
       <c r="AA62" s="16"/>
       <c r="AB62" s="16"/>
-      <c r="AC62" s="18">
+      <c r="AC62" s="16"/>
+      <c r="AD62" s="16"/>
+      <c r="AE62" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD62" s="16"/>
-      <c r="AE62" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF62" s="24"/>
+      <c r="AF62" s="16"/>
+      <c r="AG62" s="16"/>
+      <c r="AH62" s="16"/>
+      <c r="AI62" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ62" s="24"/>
     </row>
-    <row r="63" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="13">
         <v>55</v>
       </c>
       <c r="C63" s="14"/>
       <c r="D63" s="14"/>
       <c r="E63" s="22"/>
-      <c r="F63" s="46"/>
+      <c r="F63" s="26"/>
       <c r="G63" s="15"/>
       <c r="H63" s="17"/>
       <c r="I63" s="20">
@@ -11104,40 +11373,44 @@
         <v>0</v>
       </c>
       <c r="P63" s="16"/>
-      <c r="Q63" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R63" s="24"/>
-      <c r="S63" s="22"/>
-      <c r="T63" s="46"/>
-      <c r="U63" s="15"/>
-      <c r="V63" s="17"/>
-      <c r="W63" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X63" s="16"/>
-      <c r="Y63" s="16"/>
+      <c r="Q63" s="16"/>
+      <c r="R63" s="16"/>
+      <c r="S63" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T63" s="24"/>
+      <c r="U63" s="22"/>
+      <c r="V63" s="26"/>
+      <c r="W63" s="15"/>
+      <c r="X63" s="17"/>
+      <c r="Y63" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z63" s="16"/>
       <c r="AA63" s="16"/>
       <c r="AB63" s="16"/>
-      <c r="AC63" s="18">
+      <c r="AC63" s="16"/>
+      <c r="AD63" s="16"/>
+      <c r="AE63" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD63" s="16"/>
-      <c r="AE63" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF63" s="24"/>
+      <c r="AF63" s="16"/>
+      <c r="AG63" s="16"/>
+      <c r="AH63" s="16"/>
+      <c r="AI63" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ63" s="24"/>
     </row>
-    <row r="64" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="13">
         <v>56</v>
       </c>
       <c r="C64" s="14"/>
       <c r="D64" s="14"/>
       <c r="E64" s="22"/>
-      <c r="F64" s="46"/>
+      <c r="F64" s="26"/>
       <c r="G64" s="15"/>
       <c r="H64" s="17"/>
       <c r="I64" s="20">
@@ -11153,40 +11426,44 @@
         <v>0</v>
       </c>
       <c r="P64" s="16"/>
-      <c r="Q64" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R64" s="24"/>
-      <c r="S64" s="22"/>
-      <c r="T64" s="46"/>
-      <c r="U64" s="15"/>
-      <c r="V64" s="17"/>
-      <c r="W64" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X64" s="16"/>
-      <c r="Y64" s="16"/>
+      <c r="Q64" s="16"/>
+      <c r="R64" s="16"/>
+      <c r="S64" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T64" s="24"/>
+      <c r="U64" s="22"/>
+      <c r="V64" s="26"/>
+      <c r="W64" s="15"/>
+      <c r="X64" s="17"/>
+      <c r="Y64" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z64" s="16"/>
       <c r="AA64" s="16"/>
       <c r="AB64" s="16"/>
-      <c r="AC64" s="18">
+      <c r="AC64" s="16"/>
+      <c r="AD64" s="16"/>
+      <c r="AE64" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD64" s="16"/>
-      <c r="AE64" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF64" s="24"/>
+      <c r="AF64" s="16"/>
+      <c r="AG64" s="16"/>
+      <c r="AH64" s="16"/>
+      <c r="AI64" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ64" s="24"/>
     </row>
-    <row r="65" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="13">
         <v>57</v>
       </c>
       <c r="C65" s="14"/>
       <c r="D65" s="14"/>
       <c r="E65" s="22"/>
-      <c r="F65" s="46"/>
+      <c r="F65" s="26"/>
       <c r="G65" s="15"/>
       <c r="H65" s="17"/>
       <c r="I65" s="20">
@@ -11202,40 +11479,44 @@
         <v>0</v>
       </c>
       <c r="P65" s="16"/>
-      <c r="Q65" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R65" s="24"/>
-      <c r="S65" s="22"/>
-      <c r="T65" s="46"/>
-      <c r="U65" s="15"/>
-      <c r="V65" s="17"/>
-      <c r="W65" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X65" s="16"/>
-      <c r="Y65" s="16"/>
+      <c r="Q65" s="16"/>
+      <c r="R65" s="16"/>
+      <c r="S65" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T65" s="24"/>
+      <c r="U65" s="22"/>
+      <c r="V65" s="26"/>
+      <c r="W65" s="15"/>
+      <c r="X65" s="17"/>
+      <c r="Y65" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z65" s="16"/>
       <c r="AA65" s="16"/>
       <c r="AB65" s="16"/>
-      <c r="AC65" s="18">
+      <c r="AC65" s="16"/>
+      <c r="AD65" s="16"/>
+      <c r="AE65" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD65" s="16"/>
-      <c r="AE65" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF65" s="24"/>
+      <c r="AF65" s="16"/>
+      <c r="AG65" s="16"/>
+      <c r="AH65" s="16"/>
+      <c r="AI65" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ65" s="24"/>
     </row>
-    <row r="66" spans="2:32" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:36" s="12" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="13">
         <v>58</v>
       </c>
       <c r="C66" s="14"/>
       <c r="D66" s="14"/>
       <c r="E66" s="22"/>
-      <c r="F66" s="46"/>
+      <c r="F66" s="26"/>
       <c r="G66" s="15"/>
       <c r="H66" s="17"/>
       <c r="I66" s="20">
@@ -11251,40 +11532,44 @@
         <v>0</v>
       </c>
       <c r="P66" s="16"/>
-      <c r="Q66" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R66" s="24"/>
-      <c r="S66" s="22"/>
-      <c r="T66" s="46"/>
-      <c r="U66" s="15"/>
-      <c r="V66" s="17"/>
-      <c r="W66" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X66" s="16"/>
-      <c r="Y66" s="16"/>
+      <c r="Q66" s="16"/>
+      <c r="R66" s="16"/>
+      <c r="S66" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T66" s="24"/>
+      <c r="U66" s="22"/>
+      <c r="V66" s="26"/>
+      <c r="W66" s="15"/>
+      <c r="X66" s="17"/>
+      <c r="Y66" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z66" s="16"/>
       <c r="AA66" s="16"/>
       <c r="AB66" s="16"/>
-      <c r="AC66" s="18">
+      <c r="AC66" s="16"/>
+      <c r="AD66" s="16"/>
+      <c r="AE66" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD66" s="16"/>
-      <c r="AE66" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF66" s="24"/>
+      <c r="AF66" s="16"/>
+      <c r="AG66" s="16"/>
+      <c r="AH66" s="16"/>
+      <c r="AI66" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ66" s="24"/>
     </row>
-    <row r="67" spans="2:32" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:36" s="12" customFormat="1" ht="125.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="13">
         <v>59</v>
       </c>
       <c r="C67" s="14"/>
       <c r="D67" s="14"/>
       <c r="E67" s="22"/>
-      <c r="F67" s="46"/>
+      <c r="F67" s="26"/>
       <c r="G67" s="15"/>
       <c r="H67" s="17"/>
       <c r="I67" s="20">
@@ -11300,43 +11585,72 @@
         <v>0</v>
       </c>
       <c r="P67" s="16"/>
-      <c r="Q67" s="19">
-        <v>20000</v>
-      </c>
-      <c r="R67" s="24"/>
-      <c r="S67" s="22"/>
-      <c r="T67" s="46"/>
-      <c r="U67" s="15"/>
-      <c r="V67" s="17"/>
-      <c r="W67" s="20">
-        <v>7.85</v>
-      </c>
-      <c r="X67" s="16"/>
-      <c r="Y67" s="16"/>
+      <c r="Q67" s="16"/>
+      <c r="R67" s="16"/>
+      <c r="S67" s="19">
+        <v>20000</v>
+      </c>
+      <c r="T67" s="24"/>
+      <c r="U67" s="22"/>
+      <c r="V67" s="26"/>
+      <c r="W67" s="15"/>
+      <c r="X67" s="17"/>
+      <c r="Y67" s="20">
+        <v>7.85</v>
+      </c>
       <c r="Z67" s="16"/>
       <c r="AA67" s="16"/>
       <c r="AB67" s="16"/>
-      <c r="AC67" s="18">
+      <c r="AC67" s="16"/>
+      <c r="AD67" s="16"/>
+      <c r="AE67" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AD67" s="16"/>
-      <c r="AE67" s="19">
-        <v>20000</v>
-      </c>
-      <c r="AF67" s="24"/>
+      <c r="AF67" s="16"/>
+      <c r="AG67" s="16"/>
+      <c r="AH67" s="16"/>
+      <c r="AI67" s="19">
+        <v>20000</v>
+      </c>
+      <c r="AJ67" s="24"/>
     </row>
   </sheetData>
-  <autoFilter ref="B6:AF67" xr:uid="{00000000-0009-0000-0000-00001B000000}"/>
-  <mergeCells count="37">
+  <autoFilter ref="B6:AJ67" xr:uid="{00000000-0009-0000-0000-00001B000000}"/>
+  <mergeCells count="41">
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="Q3:Q5"/>
+    <mergeCell ref="R3:R5"/>
+    <mergeCell ref="AJ2:AJ5"/>
+    <mergeCell ref="AD3:AD5"/>
+    <mergeCell ref="P3:P5"/>
+    <mergeCell ref="U1:AJ1"/>
+    <mergeCell ref="AI2:AI5"/>
+    <mergeCell ref="X3:X5"/>
+    <mergeCell ref="Z4:Z5"/>
+    <mergeCell ref="AA4:AA5"/>
+    <mergeCell ref="AC4:AC5"/>
+    <mergeCell ref="AB4:AB5"/>
+    <mergeCell ref="AF3:AF5"/>
+    <mergeCell ref="Z3:AC3"/>
+    <mergeCell ref="U2:AF2"/>
+    <mergeCell ref="AG3:AG5"/>
+    <mergeCell ref="AH3:AH5"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="U3:U5"/>
+    <mergeCell ref="Y3:Y5"/>
+    <mergeCell ref="AE3:AE5"/>
+    <mergeCell ref="W3:W5"/>
     <mergeCell ref="K4:K5"/>
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="M4:M5"/>
-    <mergeCell ref="T3:T5"/>
-    <mergeCell ref="E1:R1"/>
+    <mergeCell ref="V3:V5"/>
+    <mergeCell ref="E1:T1"/>
     <mergeCell ref="E2:P2"/>
-    <mergeCell ref="Q2:Q5"/>
-    <mergeCell ref="R2:R5"/>
+    <mergeCell ref="S2:S5"/>
+    <mergeCell ref="T2:T5"/>
     <mergeCell ref="E3:E5"/>
     <mergeCell ref="F3:F5"/>
     <mergeCell ref="G3:G5"/>
@@ -11345,27 +11659,6 @@
     <mergeCell ref="J3:M3"/>
     <mergeCell ref="N3:N5"/>
     <mergeCell ref="O3:O5"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="S3:S5"/>
-    <mergeCell ref="W3:W5"/>
-    <mergeCell ref="AC3:AC5"/>
-    <mergeCell ref="U3:U5"/>
-    <mergeCell ref="AF2:AF5"/>
-    <mergeCell ref="AB3:AB5"/>
-    <mergeCell ref="P3:P5"/>
-    <mergeCell ref="S1:AF1"/>
-    <mergeCell ref="AE2:AE5"/>
-    <mergeCell ref="V3:V5"/>
-    <mergeCell ref="X4:X5"/>
-    <mergeCell ref="Y4:Y5"/>
-    <mergeCell ref="AA4:AA5"/>
-    <mergeCell ref="Z4:Z5"/>
-    <mergeCell ref="AD3:AD5"/>
-    <mergeCell ref="X3:AA3"/>
-    <mergeCell ref="S2:AD2"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="D2:D5"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
fix logic weight excel
</commit_message>
<xml_diff>
--- a/app/templates/VAVE_Analysis_Import_Template.xlsx
+++ b/app/templates/VAVE_Analysis_Import_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WebSource\PROMISE-APPS\promise-inventory\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C998871E-B8D1-478B-9918-72F31A92B1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87777DD2-2CF9-4A7B-8C74-5492C4BDD6C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{62AADBC6-8410-49F7-A504-0FB573E6F6A1}"/>
   </bookViews>
@@ -1458,7 +1458,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1469,13 +1469,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="15" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1487,21 +1493,6 @@
     <xf numFmtId="15" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1509,6 +1500,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1611,7 +1611,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="32504063" y="20926425"/>
+          <a:off x="33027938" y="20926425"/>
           <a:ext cx="0" cy="1504279"/>
           <a:chOff x="63665100" y="150342600"/>
           <a:chExt cx="1016508" cy="908966"/>
@@ -1742,7 +1742,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="32504063" y="11353800"/>
+          <a:off x="33027938" y="11353800"/>
           <a:ext cx="0" cy="1504279"/>
           <a:chOff x="63665100" y="150342600"/>
           <a:chExt cx="1016508" cy="908966"/>
@@ -8067,7 +8067,9 @@
     <col min="10" max="10" width="16.5546875" style="1" customWidth="1"/>
     <col min="11" max="12" width="20.6640625" style="1" customWidth="1"/>
     <col min="13" max="13" width="21.5546875" style="1" customWidth="1"/>
-    <col min="14" max="18" width="14.5546875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="14.5546875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="22.33203125" style="1" customWidth="1"/>
+    <col min="16" max="18" width="14.5546875" style="1" customWidth="1"/>
     <col min="19" max="19" width="17.88671875" style="1" customWidth="1"/>
     <col min="20" max="20" width="27.88671875" style="1" customWidth="1"/>
     <col min="21" max="22" width="34.6640625" style="2" customWidth="1"/>
@@ -8087,44 +8089,44 @@
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="31" t="s">
+      <c r="E1" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="M1" s="31"/>
-      <c r="N1" s="31"/>
-      <c r="O1" s="31"/>
-      <c r="P1" s="31"/>
-      <c r="Q1" s="31"/>
-      <c r="R1" s="31"/>
-      <c r="S1" s="31"/>
-      <c r="T1" s="31"/>
-      <c r="U1" s="31"/>
-      <c r="V1" s="31"/>
-      <c r="W1" s="31"/>
-      <c r="X1" s="31"/>
-      <c r="Y1" s="31"/>
-      <c r="Z1" s="31"/>
-      <c r="AA1" s="31"/>
-      <c r="AB1" s="31"/>
-      <c r="AC1" s="31"/>
-      <c r="AD1" s="31"/>
-      <c r="AE1" s="31"/>
-      <c r="AF1" s="31"/>
-      <c r="AG1" s="31"/>
-      <c r="AH1" s="31"/>
-      <c r="AI1" s="31"/>
-      <c r="AJ1" s="31"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+      <c r="U1" s="35"/>
+      <c r="V1" s="35"/>
+      <c r="W1" s="35"/>
+      <c r="X1" s="35"/>
+      <c r="Y1" s="35"/>
+      <c r="Z1" s="35"/>
+      <c r="AA1" s="35"/>
+      <c r="AB1" s="35"/>
+      <c r="AC1" s="35"/>
+      <c r="AD1" s="35"/>
+      <c r="AE1" s="35"/>
+      <c r="AF1" s="35"/>
+      <c r="AG1" s="35"/>
+      <c r="AH1" s="35"/>
+      <c r="AI1" s="35"/>
+      <c r="AJ1" s="35"/>
     </row>
     <row r="2" spans="1:36" s="5" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="27" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="28" t="s">
@@ -8133,220 +8135,220 @@
       <c r="D2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="32"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33"/>
-      <c r="K2" s="33"/>
-      <c r="L2" s="33"/>
-      <c r="M2" s="33"/>
-      <c r="N2" s="33"/>
-      <c r="O2" s="33"/>
-      <c r="P2" s="33"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
+      <c r="N2" s="43"/>
+      <c r="O2" s="43"/>
+      <c r="P2" s="43"/>
       <c r="Q2" s="25"/>
       <c r="R2" s="25"/>
-      <c r="S2" s="34" t="s">
+      <c r="S2" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="T2" s="37" t="s">
+      <c r="T2" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="32"/>
-      <c r="V2" s="33"/>
-      <c r="W2" s="33"/>
-      <c r="X2" s="33"/>
-      <c r="Y2" s="33"/>
-      <c r="Z2" s="33"/>
-      <c r="AA2" s="33"/>
-      <c r="AB2" s="33"/>
-      <c r="AC2" s="33"/>
-      <c r="AD2" s="33"/>
-      <c r="AE2" s="33"/>
-      <c r="AF2" s="33"/>
+      <c r="U2" s="42"/>
+      <c r="V2" s="43"/>
+      <c r="W2" s="43"/>
+      <c r="X2" s="43"/>
+      <c r="Y2" s="43"/>
+      <c r="Z2" s="43"/>
+      <c r="AA2" s="43"/>
+      <c r="AB2" s="43"/>
+      <c r="AC2" s="43"/>
+      <c r="AD2" s="43"/>
+      <c r="AE2" s="43"/>
+      <c r="AF2" s="43"/>
       <c r="AG2" s="25"/>
       <c r="AH2" s="25"/>
-      <c r="AI2" s="34" t="s">
+      <c r="AI2" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="AJ2" s="37" t="s">
+      <c r="AJ2" s="32" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:36" s="5" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
-      <c r="B3" s="41"/>
+      <c r="B3" s="27"/>
       <c r="C3" s="29"/>
       <c r="D3" s="29"/>
-      <c r="E3" s="40" t="s">
+      <c r="E3" s="44" t="s">
         <v>15</v>
       </c>
       <c r="F3" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="41" t="s">
+      <c r="G3" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="42" t="s">
+      <c r="H3" s="39" t="s">
         <v>14</v>
       </c>
       <c r="I3" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="41" t="s">
+      <c r="J3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="41"/>
-      <c r="L3" s="41"/>
-      <c r="M3" s="41"/>
-      <c r="N3" s="27" t="s">
+      <c r="K3" s="27"/>
+      <c r="L3" s="27"/>
+      <c r="M3" s="27"/>
+      <c r="N3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="O3" s="27" t="s">
+      <c r="O3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="P3" s="27" t="s">
+      <c r="P3" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="Q3" s="27" t="s">
+      <c r="Q3" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="27" t="s">
+      <c r="R3" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="S3" s="35"/>
-      <c r="T3" s="38"/>
-      <c r="U3" s="40" t="s">
+      <c r="S3" s="37"/>
+      <c r="T3" s="33"/>
+      <c r="U3" s="44" t="s">
         <v>18</v>
       </c>
       <c r="V3" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="W3" s="41" t="s">
+      <c r="W3" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="X3" s="42" t="s">
+      <c r="X3" s="39" t="s">
         <v>14</v>
       </c>
       <c r="Y3" s="45" t="s">
         <v>9</v>
       </c>
-      <c r="Z3" s="41" t="s">
+      <c r="Z3" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="AA3" s="41"/>
-      <c r="AB3" s="41"/>
-      <c r="AC3" s="41"/>
-      <c r="AD3" s="27" t="s">
+      <c r="AA3" s="27"/>
+      <c r="AB3" s="27"/>
+      <c r="AC3" s="27"/>
+      <c r="AD3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="AE3" s="27" t="s">
+      <c r="AE3" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="AF3" s="27" t="s">
+      <c r="AF3" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="AG3" s="27" t="s">
+      <c r="AG3" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="AH3" s="27" t="s">
+      <c r="AH3" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="AI3" s="35"/>
-      <c r="AJ3" s="38"/>
+      <c r="AI3" s="37"/>
+      <c r="AJ3" s="33"/>
     </row>
     <row r="4" spans="1:36" s="5" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="B4" s="41"/>
+      <c r="B4" s="27"/>
       <c r="C4" s="29"/>
       <c r="D4" s="29"/>
-      <c r="E4" s="40"/>
+      <c r="E4" s="44"/>
       <c r="F4" s="29"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="43"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="40"/>
       <c r="I4" s="46"/>
-      <c r="J4" s="27" t="s">
+      <c r="J4" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="27" t="s">
+      <c r="K4" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="27" t="s">
+      <c r="L4" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="M4" s="27" t="s">
+      <c r="M4" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
-      <c r="R4" s="27"/>
-      <c r="S4" s="35"/>
-      <c r="T4" s="38"/>
-      <c r="U4" s="40"/>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="31"/>
+      <c r="R4" s="31"/>
+      <c r="S4" s="37"/>
+      <c r="T4" s="33"/>
+      <c r="U4" s="44"/>
       <c r="V4" s="29"/>
-      <c r="W4" s="41"/>
-      <c r="X4" s="43"/>
+      <c r="W4" s="27"/>
+      <c r="X4" s="40"/>
       <c r="Y4" s="46"/>
-      <c r="Z4" s="27" t="s">
+      <c r="Z4" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="AA4" s="27" t="s">
+      <c r="AA4" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="AB4" s="27" t="s">
+      <c r="AB4" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="AC4" s="27" t="s">
+      <c r="AC4" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="AD4" s="27"/>
-      <c r="AE4" s="27"/>
-      <c r="AF4" s="27"/>
-      <c r="AG4" s="27"/>
-      <c r="AH4" s="27"/>
-      <c r="AI4" s="35"/>
-      <c r="AJ4" s="38"/>
+      <c r="AD4" s="31"/>
+      <c r="AE4" s="31"/>
+      <c r="AF4" s="31"/>
+      <c r="AG4" s="31"/>
+      <c r="AH4" s="31"/>
+      <c r="AI4" s="37"/>
+      <c r="AJ4" s="33"/>
     </row>
     <row r="5" spans="1:36" s="5" customFormat="1" ht="99.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="B5" s="41"/>
+      <c r="B5" s="27"/>
       <c r="C5" s="30"/>
       <c r="D5" s="30"/>
-      <c r="E5" s="40"/>
+      <c r="E5" s="44"/>
       <c r="F5" s="30"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="44"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="41"/>
       <c r="I5" s="47"/>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="27"/>
-      <c r="M5" s="27"/>
-      <c r="N5" s="27"/>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="27"/>
-      <c r="S5" s="36"/>
-      <c r="T5" s="39"/>
-      <c r="U5" s="40"/>
+      <c r="J5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="31"/>
+      <c r="Q5" s="31"/>
+      <c r="R5" s="31"/>
+      <c r="S5" s="38"/>
+      <c r="T5" s="34"/>
+      <c r="U5" s="44"/>
       <c r="V5" s="30"/>
-      <c r="W5" s="41"/>
-      <c r="X5" s="44"/>
+      <c r="W5" s="27"/>
+      <c r="X5" s="41"/>
       <c r="Y5" s="47"/>
-      <c r="Z5" s="27"/>
-      <c r="AA5" s="27"/>
-      <c r="AB5" s="27"/>
-      <c r="AC5" s="27"/>
-      <c r="AD5" s="27"/>
-      <c r="AE5" s="27"/>
-      <c r="AF5" s="27"/>
-      <c r="AG5" s="27"/>
-      <c r="AH5" s="27"/>
-      <c r="AI5" s="36"/>
-      <c r="AJ5" s="39"/>
+      <c r="Z5" s="31"/>
+      <c r="AA5" s="31"/>
+      <c r="AB5" s="31"/>
+      <c r="AC5" s="31"/>
+      <c r="AD5" s="31"/>
+      <c r="AE5" s="31"/>
+      <c r="AF5" s="31"/>
+      <c r="AG5" s="31"/>
+      <c r="AH5" s="31"/>
+      <c r="AI5" s="38"/>
+      <c r="AJ5" s="34"/>
     </row>
     <row r="6" spans="1:36" s="5" customFormat="1" ht="52.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
@@ -8405,7 +8407,7 @@
       <c r="M7" s="16"/>
       <c r="N7" s="16"/>
       <c r="O7" s="18">
-        <f>IF(ISNUMBER(SEARCH("coil", H7)), (J7*K7*N7*I7)/1000000, IF(ISNUMBER(SEARCH("trapezoid", H7)), (J7*K7*((L7+M7)/2)*I7)/1000000, (J7*K7*L7*I7)/1000000))</f>
+        <f>IF(ISNUMBER(SEARCH("coil", H7)), (J7*K7*N7*I7/1000000)/MAX(1, Q7), IF(ISNUMBER(SEARCH("trapezoid", H7)), (J7*K7*((L7+M7)/2)*I7/1000000)/MAX(1, R7), (J7*K7*L7*I7/1000000)/MAX(1, R7)))</f>
         <v>0</v>
       </c>
       <c r="P7" s="16"/>
@@ -8427,9 +8429,9 @@
       <c r="AB7" s="16"/>
       <c r="AC7" s="16"/>
       <c r="AD7" s="16"/>
-      <c r="AE7" s="18">
-        <f>IF(ISNUMBER(SEARCH("coil", X7)), (Z7*AA7*AD7*Y7)/1000000, IF(ISNUMBER(SEARCH("trapezoid", X7)), (Z7*AA7*((AB7+AC7)/2)*Y7)/1000000, (Z7*AA7*AB7*Y7)/1000000))</f>
-        <v>0</v>
+      <c r="AE7" s="18" t="e">
+        <f>IF(ISNUMBER(SEARCH("coil", X7)), (Z7*AA7*AD7*Y7/1000000)/AG7, IF(ISNUMBER(SEARCH("trapezoid", X7)), (Z7*AA7*((AB7+AC7)/2)*Y7/1000000)/AH7, (Z7*AA7*AB7*Y7/1000000)/AH7))</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="AF7" s="16"/>
       <c r="AG7" s="16"/>
@@ -8458,7 +8460,7 @@
       <c r="M8" s="16"/>
       <c r="N8" s="16"/>
       <c r="O8" s="18">
-        <f t="shared" ref="O8:O67" si="0">IF(ISNUMBER(SEARCH("coil", H8)), (J8*K8*N8*I8)/1000000, IF(ISNUMBER(SEARCH("trapezoid", H8)), (J8*K8*((L8+M8)/2)*I8)/1000000, (J8*K8*L8*I8)/1000000))</f>
+        <f t="shared" ref="O8:O67" si="0">IF(ISNUMBER(SEARCH("coil", H8)), (J8*K8*N8*I8/1000000)/MAX(1, Q8), IF(ISNUMBER(SEARCH("trapezoid", H8)), (J8*K8*((L8+M8)/2)*I8/1000000)/MAX(1, R8), (J8*K8*L8*I8/1000000)/MAX(1, R8)))</f>
         <v>0</v>
       </c>
       <c r="P8" s="16"/>
@@ -8480,9 +8482,9 @@
       <c r="AB8" s="16"/>
       <c r="AC8" s="16"/>
       <c r="AD8" s="16"/>
-      <c r="AE8" s="18">
-        <f t="shared" ref="AE8:AE67" si="1">IF(ISNUMBER(SEARCH("coil", X8)), (Z8*AA8*AD8*Y8)/1000000, IF(ISNUMBER(SEARCH("trapezoid", X8)), (Z8*AA8*((AB8+AC8)/2)*Y8)/1000000, (Z8*AA8*AB8*Y8)/1000000))</f>
-        <v>0</v>
+      <c r="AE8" s="18" t="e">
+        <f t="shared" ref="AE8:AE67" si="1">IF(ISNUMBER(SEARCH("coil", X8)), (Z8*AA8*AD8*Y8/1000000)/AG8, IF(ISNUMBER(SEARCH("trapezoid", X8)), (Z8*AA8*((AB8+AC8)/2)*Y8/1000000)/AH8, (Z8*AA8*AB8*Y8/1000000)/AH8))</f>
+        <v>#DIV/0!</v>
       </c>
       <c r="AF8" s="16"/>
       <c r="AG8" s="16"/>
@@ -8533,9 +8535,9 @@
       <c r="AB9" s="16"/>
       <c r="AC9" s="16"/>
       <c r="AD9" s="16"/>
-      <c r="AE9" s="18">
+      <c r="AE9" s="18" t="e">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="AF9" s="16"/>
       <c r="AG9" s="16"/>
@@ -8587,7 +8589,7 @@
       <c r="AC10" s="16"/>
       <c r="AD10" s="16"/>
       <c r="AE10" s="18">
-        <f t="shared" si="1"/>
+        <f>IF(ISNUMBER(SEARCH("coil", X10)), (Z10*AA10*AD10*Y10/1000000)/MAX(1, AG10), IF(ISNUMBER(SEARCH("trapezoid", X10)), (Z10*AA10*((AB10+AC10)/2)*Y10/1000000)/MAX(1, AH10), (Z10*AA10*AB10*Y10/1000000)/MAX(1, AH10)))</f>
         <v>0</v>
       </c>
       <c r="AF10" s="16"/>
@@ -8640,7 +8642,7 @@
       <c r="AC11" s="16"/>
       <c r="AD11" s="16"/>
       <c r="AE11" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="AE11:AE67" si="2">IF(ISNUMBER(SEARCH("coil", X11)), (Z11*AA11*AD11*Y11/1000000)/MAX(1, AG11), IF(ISNUMBER(SEARCH("trapezoid", X11)), (Z11*AA11*((AB11+AC11)/2)*Y11/1000000)/MAX(1, AH11), (Z11*AA11*AB11*Y11/1000000)/MAX(1, AH11)))</f>
         <v>0</v>
       </c>
       <c r="AF11" s="16"/>
@@ -8693,7 +8695,7 @@
       <c r="AC12" s="16"/>
       <c r="AD12" s="16"/>
       <c r="AE12" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF12" s="16"/>
@@ -8746,7 +8748,7 @@
       <c r="AC13" s="16"/>
       <c r="AD13" s="16"/>
       <c r="AE13" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF13" s="16"/>
@@ -8799,7 +8801,7 @@
       <c r="AC14" s="16"/>
       <c r="AD14" s="16"/>
       <c r="AE14" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF14" s="16"/>
@@ -8852,7 +8854,7 @@
       <c r="AC15" s="16"/>
       <c r="AD15" s="16"/>
       <c r="AE15" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF15" s="16"/>
@@ -8905,7 +8907,7 @@
       <c r="AC16" s="16"/>
       <c r="AD16" s="16"/>
       <c r="AE16" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF16" s="16"/>
@@ -8958,7 +8960,7 @@
       <c r="AC17" s="16"/>
       <c r="AD17" s="16"/>
       <c r="AE17" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF17" s="16"/>
@@ -9011,7 +9013,7 @@
       <c r="AC18" s="16"/>
       <c r="AD18" s="16"/>
       <c r="AE18" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF18" s="16"/>
@@ -9064,7 +9066,7 @@
       <c r="AC19" s="16"/>
       <c r="AD19" s="16"/>
       <c r="AE19" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF19" s="16"/>
@@ -9115,7 +9117,7 @@
       <c r="AC20" s="16"/>
       <c r="AD20" s="16"/>
       <c r="AE20" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF20" s="16"/>
@@ -9168,7 +9170,7 @@
       <c r="AC21" s="16"/>
       <c r="AD21" s="16"/>
       <c r="AE21" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF21" s="16"/>
@@ -9221,7 +9223,7 @@
       <c r="AC22" s="16"/>
       <c r="AD22" s="16"/>
       <c r="AE22" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF22" s="16"/>
@@ -9274,7 +9276,7 @@
       <c r="AC23" s="16"/>
       <c r="AD23" s="16"/>
       <c r="AE23" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF23" s="16"/>
@@ -9327,7 +9329,7 @@
       <c r="AC24" s="16"/>
       <c r="AD24" s="16"/>
       <c r="AE24" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF24" s="16"/>
@@ -9380,7 +9382,7 @@
       <c r="AC25" s="16"/>
       <c r="AD25" s="16"/>
       <c r="AE25" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF25" s="16"/>
@@ -9433,7 +9435,7 @@
       <c r="AC26" s="16"/>
       <c r="AD26" s="16"/>
       <c r="AE26" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF26" s="16"/>
@@ -9486,7 +9488,7 @@
       <c r="AC27" s="16"/>
       <c r="AD27" s="16"/>
       <c r="AE27" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF27" s="16"/>
@@ -9539,7 +9541,7 @@
       <c r="AC28" s="16"/>
       <c r="AD28" s="16"/>
       <c r="AE28" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF28" s="16"/>
@@ -9590,7 +9592,7 @@
       <c r="AC29" s="16"/>
       <c r="AD29" s="16"/>
       <c r="AE29" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF29" s="16"/>
@@ -9643,7 +9645,7 @@
       <c r="AC30" s="16"/>
       <c r="AD30" s="16"/>
       <c r="AE30" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF30" s="16"/>
@@ -9696,7 +9698,7 @@
       <c r="AC31" s="16"/>
       <c r="AD31" s="16"/>
       <c r="AE31" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF31" s="16"/>
@@ -9749,7 +9751,7 @@
       <c r="AC32" s="16"/>
       <c r="AD32" s="16"/>
       <c r="AE32" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF32" s="16"/>
@@ -9802,7 +9804,7 @@
       <c r="AC33" s="16"/>
       <c r="AD33" s="16"/>
       <c r="AE33" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF33" s="16"/>
@@ -9855,7 +9857,7 @@
       <c r="AC34" s="16"/>
       <c r="AD34" s="16"/>
       <c r="AE34" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF34" s="16"/>
@@ -9908,7 +9910,7 @@
       <c r="AC35" s="16"/>
       <c r="AD35" s="16"/>
       <c r="AE35" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF35" s="16"/>
@@ -9961,7 +9963,7 @@
       <c r="AC36" s="16"/>
       <c r="AD36" s="16"/>
       <c r="AE36" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF36" s="16"/>
@@ -10014,7 +10016,7 @@
       <c r="AC37" s="16"/>
       <c r="AD37" s="16"/>
       <c r="AE37" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF37" s="16"/>
@@ -10067,7 +10069,7 @@
       <c r="AC38" s="16"/>
       <c r="AD38" s="16"/>
       <c r="AE38" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF38" s="16"/>
@@ -10120,7 +10122,7 @@
       <c r="AC39" s="16"/>
       <c r="AD39" s="16"/>
       <c r="AE39" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF39" s="16"/>
@@ -10173,7 +10175,7 @@
       <c r="AC40" s="16"/>
       <c r="AD40" s="16"/>
       <c r="AE40" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF40" s="16"/>
@@ -10226,7 +10228,7 @@
       <c r="AC41" s="16"/>
       <c r="AD41" s="16"/>
       <c r="AE41" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF41" s="16"/>
@@ -10279,7 +10281,7 @@
       <c r="AC42" s="16"/>
       <c r="AD42" s="16"/>
       <c r="AE42" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF42" s="16"/>
@@ -10332,7 +10334,7 @@
       <c r="AC43" s="16"/>
       <c r="AD43" s="16"/>
       <c r="AE43" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF43" s="16"/>
@@ -10385,7 +10387,7 @@
       <c r="AC44" s="16"/>
       <c r="AD44" s="16"/>
       <c r="AE44" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF44" s="16"/>
@@ -10438,7 +10440,7 @@
       <c r="AC45" s="16"/>
       <c r="AD45" s="16"/>
       <c r="AE45" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF45" s="16"/>
@@ -10491,7 +10493,7 @@
       <c r="AC46" s="16"/>
       <c r="AD46" s="16"/>
       <c r="AE46" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF46" s="16"/>
@@ -10544,7 +10546,7 @@
       <c r="AC47" s="16"/>
       <c r="AD47" s="16"/>
       <c r="AE47" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF47" s="16"/>
@@ -10597,7 +10599,7 @@
       <c r="AC48" s="16"/>
       <c r="AD48" s="16"/>
       <c r="AE48" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF48" s="16"/>
@@ -10650,7 +10652,7 @@
       <c r="AC49" s="16"/>
       <c r="AD49" s="16"/>
       <c r="AE49" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF49" s="16"/>
@@ -10703,7 +10705,7 @@
       <c r="AC50" s="16"/>
       <c r="AD50" s="16"/>
       <c r="AE50" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF50" s="16"/>
@@ -10756,7 +10758,7 @@
       <c r="AC51" s="16"/>
       <c r="AD51" s="16"/>
       <c r="AE51" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF51" s="16"/>
@@ -10809,7 +10811,7 @@
       <c r="AC52" s="16"/>
       <c r="AD52" s="16"/>
       <c r="AE52" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF52" s="16"/>
@@ -10862,7 +10864,7 @@
       <c r="AC53" s="16"/>
       <c r="AD53" s="16"/>
       <c r="AE53" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF53" s="16"/>
@@ -10915,7 +10917,7 @@
       <c r="AC54" s="16"/>
       <c r="AD54" s="16"/>
       <c r="AE54" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF54" s="16"/>
@@ -10968,7 +10970,7 @@
       <c r="AC55" s="16"/>
       <c r="AD55" s="16"/>
       <c r="AE55" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF55" s="16"/>
@@ -11021,7 +11023,7 @@
       <c r="AC56" s="16"/>
       <c r="AD56" s="16"/>
       <c r="AE56" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF56" s="16"/>
@@ -11074,7 +11076,7 @@
       <c r="AC57" s="16"/>
       <c r="AD57" s="16"/>
       <c r="AE57" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF57" s="16"/>
@@ -11127,7 +11129,7 @@
       <c r="AC58" s="16"/>
       <c r="AD58" s="16"/>
       <c r="AE58" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF58" s="16"/>
@@ -11180,7 +11182,7 @@
       <c r="AC59" s="16"/>
       <c r="AD59" s="16"/>
       <c r="AE59" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF59" s="16"/>
@@ -11233,7 +11235,7 @@
       <c r="AC60" s="16"/>
       <c r="AD60" s="16"/>
       <c r="AE60" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF60" s="16"/>
@@ -11286,7 +11288,7 @@
       <c r="AC61" s="16"/>
       <c r="AD61" s="16"/>
       <c r="AE61" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF61" s="16"/>
@@ -11339,7 +11341,7 @@
       <c r="AC62" s="16"/>
       <c r="AD62" s="16"/>
       <c r="AE62" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF62" s="16"/>
@@ -11392,7 +11394,7 @@
       <c r="AC63" s="16"/>
       <c r="AD63" s="16"/>
       <c r="AE63" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF63" s="16"/>
@@ -11445,7 +11447,7 @@
       <c r="AC64" s="16"/>
       <c r="AD64" s="16"/>
       <c r="AE64" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF64" s="16"/>
@@ -11498,7 +11500,7 @@
       <c r="AC65" s="16"/>
       <c r="AD65" s="16"/>
       <c r="AE65" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF65" s="16"/>
@@ -11551,7 +11553,7 @@
       <c r="AC66" s="16"/>
       <c r="AD66" s="16"/>
       <c r="AE66" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF66" s="16"/>
@@ -11604,7 +11606,7 @@
       <c r="AC67" s="16"/>
       <c r="AD67" s="16"/>
       <c r="AE67" s="18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF67" s="16"/>
@@ -11618,11 +11620,25 @@
   </sheetData>
   <autoFilter ref="B6:AJ67" xr:uid="{00000000-0009-0000-0000-00001B000000}"/>
   <mergeCells count="41">
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="Q3:Q5"/>
-    <mergeCell ref="R3:R5"/>
+    <mergeCell ref="E1:T1"/>
+    <mergeCell ref="E2:P2"/>
+    <mergeCell ref="S2:S5"/>
+    <mergeCell ref="T2:T5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="F3:F5"/>
+    <mergeCell ref="G3:G5"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="N3:N5"/>
+    <mergeCell ref="O3:O5"/>
+    <mergeCell ref="Y3:Y5"/>
+    <mergeCell ref="AE3:AE5"/>
+    <mergeCell ref="W3:W5"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="V3:V5"/>
     <mergeCell ref="AJ2:AJ5"/>
     <mergeCell ref="AD3:AD5"/>
     <mergeCell ref="P3:P5"/>
@@ -11638,27 +11654,13 @@
     <mergeCell ref="U2:AF2"/>
     <mergeCell ref="AG3:AG5"/>
     <mergeCell ref="AH3:AH5"/>
+    <mergeCell ref="U3:U5"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="Q3:Q5"/>
+    <mergeCell ref="R3:R5"/>
     <mergeCell ref="J4:J5"/>
-    <mergeCell ref="U3:U5"/>
-    <mergeCell ref="Y3:Y5"/>
-    <mergeCell ref="AE3:AE5"/>
-    <mergeCell ref="W3:W5"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="M4:M5"/>
-    <mergeCell ref="V3:V5"/>
-    <mergeCell ref="E1:T1"/>
-    <mergeCell ref="E2:P2"/>
-    <mergeCell ref="S2:S5"/>
-    <mergeCell ref="T2:T5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="F3:F5"/>
-    <mergeCell ref="G3:G5"/>
-    <mergeCell ref="H3:H5"/>
-    <mergeCell ref="I3:I5"/>
-    <mergeCell ref="J3:M3"/>
-    <mergeCell ref="N3:N5"/>
-    <mergeCell ref="O3:O5"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>